<commit_message>
Implement Leave Monetization Candidates page and related functionality. Added a new page for displaying leave monetization candidates, including filtering, sorting, and pagination features. Introduced a verification script for smoke testing monetization candidates data. Updated the leader tracker with new task statuses and completion details, and adjusted the date for the last code sync.
</commit_message>
<xml_diff>
--- a/docs/FRONTEND_LEADER_TRACKER.xlsx
+++ b/docs/FRONTEND_LEADER_TRACKER.xlsx
@@ -131,11 +131,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
@@ -146,17 +141,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E2D5F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
@@ -213,22 +213,22 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="9" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -248,6 +248,13 @@
     <xf numFmtId="9" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -267,13 +274,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -297,17 +297,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -321,7 +321,7 @@
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -333,11 +333,11 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -751,7 +751,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Last aligned to codebase: 2026-07-23 — employee and approver/team UIs are largely built with mock data; team calendar/upcoming and admin routes are still placeholders; cookie/session and live API are not wired yet.</t>
+          <t>Last aligned to codebase: 2026-07-29 — all employee, approver/team, and admin screens now have real UI with mock data; 2 minor report sub-pages still placeholders; cookie/session and live API not wired yet.</t>
         </is>
       </c>
     </row>
@@ -1877,15 +1877,15 @@
         <v>46225</v>
       </c>
       <c r="D7" s="50" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="E7" s="18">
         <f>IF(OR(C7="",D7=""),"",NETWORKDAYS(C7,D7))</f>
         <v/>
       </c>
-      <c r="F7" s="61" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G7" s="19">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="I7" s="49" t="inlineStr">
         <is>
-          <t>Done so far: StatusBadge, FilterSelect, Pagination, LeaveTypeIconBadge, Modal, ConfirmReasonModal, AttachmentPreviewModal, and form fields. Full shared button/table kit still pending.</t>
+          <t>Built: StatusBadge, FilterSelect, Pagination, Button, Modal, ConfirmReasonModal, AttachmentPreviewModal, SuccessDialog, Skeleton, form fields, MonthYearPickerField, EmployeeMultiSelect, tableStyles, admin-specific components.</t>
         </is>
       </c>
     </row>
@@ -1917,15 +1917,15 @@
         <v>46225</v>
       </c>
       <c r="D8" s="50" t="n">
-        <v>46262</v>
+        <v>46232</v>
       </c>
       <c r="E8" s="18">
         <f>IF(OR(C8="",D8=""),"",NETWORKDAYS(C8,D8))</f>
         <v/>
       </c>
-      <c r="F8" s="61" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G8" s="19">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="I8" s="49" t="inlineStr">
         <is>
-          <t>Real pages now cover employee + key approver/team flows. Team calendar/upcoming and all admin routes still use PagePlaceholder.</t>
+          <t>All employee, approver/team, and admin routes now have real page components. No PagePlaceholder routes remain (only 2 minor sub-reports still placeholders).</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
         <f>IF(F9="Completed",1,IF(F9="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H9" s="62">
+      <c r="H9" s="61">
         <f>IF(C9="","",C9+MOD(5-WEEKDAY(C9,2),7))</f>
         <v/>
       </c>
@@ -2012,7 +2012,7 @@
         <f>IF(F10="Completed",1,IF(F10="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H10" s="62">
+      <c r="H10" s="61">
         <f>IF(C10="","",C10+MOD(5-WEEKDAY(C10,2),7))</f>
         <v/>
       </c>
@@ -2052,7 +2052,7 @@
         <f>IF(F11="Completed",1,IF(F11="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H11" s="62">
+      <c r="H11" s="61">
         <f>IF(C11="","",C11+MOD(5-WEEKDAY(C11,2),7))</f>
         <v/>
       </c>
@@ -2092,7 +2092,7 @@
         <f>IF(F12="Completed",1,IF(F12="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H12" s="62">
+      <c r="H12" s="61">
         <f>IF(C12="","",C12+MOD(5-WEEKDAY(C12,2),7))</f>
         <v/>
       </c>
@@ -2132,7 +2132,7 @@
         <f>IF(F13="Completed",1,IF(F13="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H13" s="62">
+      <c r="H13" s="61">
         <f>IF(C13="","",C13+MOD(5-WEEKDAY(C13,2),7))</f>
         <v/>
       </c>
@@ -2172,7 +2172,7 @@
         <f>IF(F14="Completed",1,IF(F14="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H14" s="62">
+      <c r="H14" s="61">
         <f>IF(C14="","",C14+MOD(5-WEEKDAY(C14,2),7))</f>
         <v/>
       </c>
@@ -2212,7 +2212,7 @@
         <f>IF(F15="Completed",1,IF(F15="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H15" s="62">
+      <c r="H15" s="61">
         <f>IF(C15="","",C15+MOD(5-WEEKDAY(C15,2),7))</f>
         <v/>
       </c>
@@ -2252,7 +2252,7 @@
         <f>IF(F16="Completed",1,IF(F16="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H16" s="62">
+      <c r="H16" s="61">
         <f>IF(C16="","",C16+MOD(5-WEEKDAY(C16,2),7))</f>
         <v/>
       </c>
@@ -2292,7 +2292,7 @@
         <f>IF(F17="Completed",1,IF(F17="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H17" s="63">
+      <c r="H17" s="62">
         <f>IF(C17="","",C17+MOD(5-WEEKDAY(C17,2),7))</f>
         <v/>
       </c>
@@ -2332,7 +2332,7 @@
         <f>IF(F18="Completed",1,IF(F18="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H18" s="63">
+      <c r="H18" s="62">
         <f>IF(C18="","",C18+MOD(5-WEEKDAY(C18,2),7))</f>
         <v/>
       </c>
@@ -2372,7 +2372,7 @@
         <f>IF(F19="Completed",1,IF(F19="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H19" s="63">
+      <c r="H19" s="62">
         <f>IF(C19="","",C19+MOD(5-WEEKDAY(C19,2),7))</f>
         <v/>
       </c>
@@ -2412,7 +2412,7 @@
         <f>IF(F20="Completed",1,IF(F20="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H20" s="63">
+      <c r="H20" s="62">
         <f>IF(C20="","",C20+MOD(5-WEEKDAY(C20,2),7))</f>
         <v/>
       </c>
@@ -2434,29 +2434,33 @@
         </is>
       </c>
       <c r="C21" s="46" t="n">
-        <v>46252</v>
+        <v>46232</v>
       </c>
       <c r="D21" s="46" t="n">
-        <v>46255</v>
+        <v>46232</v>
       </c>
       <c r="E21" s="24">
         <f>IF(OR(C21="",D21=""),"",NETWORKDAYS(C21,D21))</f>
         <v/>
       </c>
-      <c r="F21" s="64" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G21" s="25">
         <f>IF(F21="Completed",1,IF(F21="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H21" s="63">
+      <c r="H21" s="62">
         <f>IF(C21="","",C21+MOD(5-WEEKDAY(C21,2),7))</f>
         <v/>
       </c>
-      <c r="I21" s="45" t="inlineStr"/>
+      <c r="I21" s="45" t="inlineStr">
+        <is>
+          <t>Team Leave Calendar page (month/week views, filters, leave chips) and Upcoming Approved Leaves page are both built with mock data.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="47" t="inlineStr">
@@ -2470,29 +2474,33 @@
         </is>
       </c>
       <c r="C22" s="48" t="n">
-        <v>46252</v>
+        <v>46232</v>
       </c>
       <c r="D22" s="48" t="n">
-        <v>46255</v>
+        <v>46232</v>
       </c>
       <c r="E22" s="27">
         <f>IF(OR(C22="",D22=""),"",NETWORKDAYS(C22,D22))</f>
         <v/>
       </c>
-      <c r="F22" s="64" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F22" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G22" s="28">
         <f>IF(F22="Completed",1,IF(F22="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H22" s="65">
+      <c r="H22" s="63">
         <f>IF(C22="","",C22+MOD(5-WEEKDAY(C22,2),7))</f>
         <v/>
       </c>
-      <c r="I22" s="47" t="inlineStr"/>
+      <c r="I22" s="47" t="inlineStr">
+        <is>
+          <t>Admin Leave Requests list (pending/all tabs, filters, search, reminders) and detail/view/validate pages are all built with mock data.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="47" t="inlineStr">
@@ -2506,29 +2514,33 @@
         </is>
       </c>
       <c r="C23" s="48" t="n">
-        <v>46254</v>
+        <v>46232</v>
       </c>
       <c r="D23" s="48" t="n">
-        <v>46259</v>
+        <v>46232</v>
       </c>
       <c r="E23" s="27">
         <f>IF(OR(C23="",D23=""),"",NETWORKDAYS(C23,D23))</f>
         <v/>
       </c>
-      <c r="F23" s="64" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F23" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G23" s="28">
         <f>IF(F23="Completed",1,IF(F23="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H23" s="65">
+      <c r="H23" s="63">
         <f>IF(C23="","",C23+MOD(5-WEEKDAY(C23,2),7))</f>
         <v/>
       </c>
-      <c r="I23" s="47" t="inlineStr"/>
+      <c r="I23" s="47" t="inlineStr">
+        <is>
+          <t>Conversion review is handled via Admin Leave Validate page; conversion state visible on request detail/view pages.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="47" t="inlineStr">
@@ -2542,29 +2554,33 @@
         </is>
       </c>
       <c r="C24" s="48" t="n">
-        <v>46254</v>
+        <v>46232</v>
       </c>
       <c r="D24" s="48" t="n">
-        <v>46260</v>
+        <v>46232</v>
       </c>
       <c r="E24" s="27">
         <f>IF(OR(C24="",D24=""),"",NETWORKDAYS(C24,D24))</f>
         <v/>
       </c>
-      <c r="F24" s="64" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F24" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G24" s="28">
         <f>IF(F24="Completed",1,IF(F24="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H24" s="65">
+      <c r="H24" s="63">
         <f>IF(C24="","",C24+MOD(5-WEEKDAY(C24,2),7))</f>
         <v/>
       </c>
-      <c r="I24" s="47" t="inlineStr"/>
+      <c r="I24" s="47" t="inlineStr">
+        <is>
+          <t>Admin Leave Balances page with filters, adjust-credits modal, and full distribution flows (annual, newly-regularized, parental, contractual) are built with mock data.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="47" t="inlineStr">
@@ -2578,29 +2594,33 @@
         </is>
       </c>
       <c r="C25" s="48" t="n">
-        <v>46259</v>
+        <v>46232</v>
       </c>
       <c r="D25" s="48" t="n">
-        <v>46261</v>
+        <v>46232</v>
       </c>
       <c r="E25" s="27">
         <f>IF(OR(C25="",D25=""),"",NETWORKDAYS(C25,D25))</f>
         <v/>
       </c>
-      <c r="F25" s="64" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F25" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G25" s="28">
         <f>IF(F25="Completed",1,IF(F25="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H25" s="65">
+      <c r="H25" s="63">
         <f>IF(C25="","",C25+MOD(5-WEEKDAY(C25,2),7))</f>
         <v/>
       </c>
-      <c r="I25" s="47" t="inlineStr"/>
+      <c r="I25" s="47" t="inlineStr">
+        <is>
+          <t>Admin Administrative Log page with search, filters, month-year picker, sorting, and pagination is built with mock data.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="47" t="inlineStr">
@@ -2614,10 +2634,10 @@
         </is>
       </c>
       <c r="C26" s="48" t="n">
-        <v>46259</v>
+        <v>46232</v>
       </c>
       <c r="D26" s="48" t="n">
-        <v>46262</v>
+        <v>46232</v>
       </c>
       <c r="E26" s="27">
         <f>IF(OR(C26="",D26=""),"",NETWORKDAYS(C26,D26))</f>
@@ -2625,18 +2645,22 @@
       </c>
       <c r="F26" s="64" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G26" s="28">
         <f>IF(F26="Completed",1,IF(F26="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H26" s="65">
+      <c r="H26" s="63">
         <f>IF(C26="","",C26+MOD(5-WEEKDAY(C26,2),7))</f>
         <v/>
       </c>
-      <c r="I26" s="47" t="inlineStr"/>
+      <c r="I26" s="47" t="inlineStr">
+        <is>
+          <t>Monthly Attendance Report page built. Leave Monetization Candidates and Employees with LWOP sub-reports are still placeholders.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="47" t="inlineStr">
@@ -2653,28 +2677,28 @@
         <v>46225</v>
       </c>
       <c r="D27" s="48" t="n">
-        <v>46262</v>
+        <v>46232</v>
       </c>
       <c r="E27" s="27">
         <f>IF(OR(C27="",D27=""),"",NETWORKDAYS(C27,D27))</f>
         <v/>
       </c>
-      <c r="F27" s="61" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="F27" s="33" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G27" s="28">
         <f>IF(F27="Completed",1,IF(F27="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H27" s="65">
+      <c r="H27" s="63">
         <f>IF(C27="","",C27+MOD(5-WEEKDAY(C27,2),7))</f>
         <v/>
       </c>
       <c r="I27" s="47" t="inlineStr">
         <is>
-          <t>Employee and team filing screens support Emergency, PTB, and Maternity/Paternity options with attachment rules. Admin screens for these types are still not built.</t>
+          <t>Emergency, PTB, Maternity/Paternity handled in employee/team filing and in admin screens. Monthly attendance report covers all leave categories including LWOP.</t>
         </is>
       </c>
     </row>
@@ -2689,15 +2713,15 @@
           <t>Connect frontend to backend API (base connection and shared data types)</t>
         </is>
       </c>
-      <c r="C28" s="66" t="n">
+      <c r="C28" s="65" t="n">
         <v>46226</v>
       </c>
-      <c r="D28" s="66" t="n"/>
+      <c r="D28" s="65" t="n"/>
       <c r="E28" s="30">
         <f>IF(OR(C28="",D28=""),"",NETWORKDAYS(C28,D28))</f>
         <v/>
       </c>
-      <c r="F28" s="64" t="inlineStr">
+      <c r="F28" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2727,15 +2751,15 @@
           <t>Use portal cookies / session to identify the user (no separate login page)</t>
         </is>
       </c>
-      <c r="C29" s="66" t="n">
+      <c r="C29" s="65" t="n">
         <v>46226</v>
       </c>
-      <c r="D29" s="66" t="n"/>
+      <c r="D29" s="65" t="n"/>
       <c r="E29" s="30">
         <f>IF(OR(C29="",D29=""),"",NETWORKDAYS(C29,D29))</f>
         <v/>
       </c>
-      <c r="F29" s="64" t="inlineStr">
+      <c r="F29" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2765,13 +2789,13 @@
           <t>Connect employee leave screens to live API (file, history, cancel, edit)</t>
         </is>
       </c>
-      <c r="C30" s="66" t="n"/>
-      <c r="D30" s="66" t="n"/>
+      <c r="C30" s="65" t="n"/>
+      <c r="D30" s="65" t="n"/>
       <c r="E30" s="30">
         <f>IF(OR(C30="",D30=""),"",NETWORKDAYS(C30,D30))</f>
         <v/>
       </c>
-      <c r="F30" s="64" t="inlineStr">
+      <c r="F30" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2801,13 +2825,13 @@
           <t>Connect approver / team screens to live API (inbox, approve, reject)</t>
         </is>
       </c>
-      <c r="C31" s="66" t="n"/>
-      <c r="D31" s="66" t="n"/>
+      <c r="C31" s="65" t="n"/>
+      <c r="D31" s="65" t="n"/>
       <c r="E31" s="30">
         <f>IF(OR(C31="",D31=""),"",NETWORKDAYS(C31,D31))</f>
         <v/>
       </c>
-      <c r="F31" s="64" t="inlineStr">
+      <c r="F31" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2837,13 +2861,13 @@
           <t>Connect admin screens to live API (balances, conversion, reports)</t>
         </is>
       </c>
-      <c r="C32" s="66" t="n"/>
-      <c r="D32" s="66" t="n"/>
+      <c r="C32" s="65" t="n"/>
+      <c r="D32" s="65" t="n"/>
       <c r="E32" s="30">
         <f>IF(OR(C32="",D32=""),"",NETWORKDAYS(C32,D32))</f>
         <v/>
       </c>
-      <c r="F32" s="64" t="inlineStr">
+      <c r="F32" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2873,13 +2897,13 @@
           <t>Joint frontend–backend smoke check once APIs are available</t>
         </is>
       </c>
-      <c r="C33" s="66" t="n"/>
-      <c r="D33" s="66" t="n"/>
+      <c r="C33" s="65" t="n"/>
+      <c r="D33" s="65" t="n"/>
       <c r="E33" s="30">
         <f>IF(OR(C33="",D33=""),"",NETWORKDAYS(C33,D33))</f>
         <v/>
       </c>
-      <c r="F33" s="64" t="inlineStr">
+      <c r="F33" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2917,7 +2941,7 @@
         <f>IF(OR(C34="",D34=""),"",NETWORKDAYS(C34,D34))</f>
         <v/>
       </c>
-      <c r="F34" s="64" t="inlineStr">
+      <c r="F34" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2955,7 +2979,7 @@
         <f>IF(OR(C35="",D35=""),"",NETWORKDAYS(C35,D35))</f>
         <v/>
       </c>
-      <c r="F35" s="64" t="inlineStr">
+      <c r="F35" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2993,7 +3017,7 @@
         <f>IF(OR(C36="",D36=""),"",NETWORKDAYS(C36,D36))</f>
         <v/>
       </c>
-      <c r="F36" s="64" t="inlineStr">
+      <c r="F36" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3031,7 +3055,7 @@
         <f>IF(OR(C37="",D37=""),"",NETWORKDAYS(C37,D37))</f>
         <v/>
       </c>
-      <c r="F37" s="64" t="inlineStr">
+      <c r="F37" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3069,7 +3093,7 @@
         <f>IF(OR(C38="",D38=""),"",NETWORKDAYS(C38,D38))</f>
         <v/>
       </c>
-      <c r="F38" s="64" t="inlineStr">
+      <c r="F38" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3107,7 +3131,7 @@
         <f>IF(OR(C39="",D39=""),"",NETWORKDAYS(C39,D39))</f>
         <v/>
       </c>
-      <c r="F39" s="64" t="inlineStr">
+      <c r="F39" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3145,7 +3169,7 @@
         <f>IF(OR(C40="",D40=""),"",NETWORKDAYS(C40,D40))</f>
         <v/>
       </c>
-      <c r="F40" s="64" t="inlineStr">
+      <c r="F40" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3183,7 +3207,7 @@
         <f>IF(OR(C41="",D41=""),"",NETWORKDAYS(C41,D41))</f>
         <v/>
       </c>
-      <c r="F41" s="64" t="inlineStr">
+      <c r="F41" s="66" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>

</xml_diff>

<commit_message>
enhance sidebar functionality, and implement sidebar collapse preference. Improved sidebar component to support collapsible functionality with user preferences stored in local storage. Updated TopHeader to include sidebar toggle button and refined layout for better user experience.
</commit_message>
<xml_diff>
--- a/docs/FRONTEND_LEADER_TRACKER.xlsx
+++ b/docs/FRONTEND_LEADER_TRACKER.xlsx
@@ -13,7 +13,7 @@
     <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Progress Tracker'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Progress Tracker'!$A$1:$I$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -102,7 +102,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -142,6 +142,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2D5F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAD1DC"/>
       </patternFill>
     </fill>
     <fill>
@@ -201,34 +206,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -269,11 +274,18 @@
     <xf numFmtId="9" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -283,15 +295,15 @@
     <xf numFmtId="9" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="10" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="10" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -307,9 +319,9 @@
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -330,22 +342,27 @@
     <xf numFmtId="165" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -715,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -751,7 +768,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Last aligned to codebase: 2026-07-29 — all employee, approver/team, and admin screens now have real UI with mock data; 2 minor report sub-pages still placeholders; cookie/session and live API not wired yet.</t>
+          <t>Last aligned to codebase: 2026-07-30 — all screens built with mock data; currently polishing CSS and layouts (section 6); cookie/session and live API not wired yet.</t>
         </is>
       </c>
     </row>
@@ -997,7 +1014,7 @@
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>6. Backend Integration (TBD)</t>
+          <t>6. UI Polish &amp; Cleanup</t>
         </is>
       </c>
       <c r="B15" s="30">
@@ -1028,7 +1045,7 @@
     <row r="16">
       <c r="A16" s="32" t="inlineStr">
         <is>
-          <t>7. Testing (after development)</t>
+          <t>7. Backend Integration (TBD)</t>
         </is>
       </c>
       <c r="B16" s="33">
@@ -1059,7 +1076,7 @@
     <row r="17">
       <c r="A17" s="35" t="inlineStr">
         <is>
-          <t>8. Documentation (after development)</t>
+          <t>8. Testing (after development)</t>
         </is>
       </c>
       <c r="B17" s="36">
@@ -1087,14 +1104,45 @@
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="38" t="inlineStr">
-        <is>
-          <t>Development progress (sections 1–5 only)</t>
-        </is>
-      </c>
-      <c r="B19" s="39">
-        <f>IF(SUM(B10:B14)=0,0,SUMPRODUCT(B10:B14,G10:G14)/SUM(B10:B14))</f>
+    <row r="18">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>9. Documentation (after development)</t>
+        </is>
+      </c>
+      <c r="B18" s="39">
+        <f>COUNTIF('Progress Tracker'!A:A,A18)</f>
+        <v/>
+      </c>
+      <c r="C18" s="39">
+        <f>COUNTIFS('Progress Tracker'!A:A,A18,'Progress Tracker'!F:F,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D18" s="39">
+        <f>COUNTIFS('Progress Tracker'!A:A,A18,'Progress Tracker'!F:F,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E18" s="39">
+        <f>COUNTIFS('Progress Tracker'!A:A,A18,'Progress Tracker'!F:F,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F18" s="39">
+        <f>COUNTIFS('Progress Tracker'!A:A,A18,'Progress Tracker'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G18" s="40">
+        <f>IF(B18=0,0,(C18+0.5*D18)/B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Development progress (sections 1–6 only)</t>
+        </is>
+      </c>
+      <c r="B20" s="42">
+        <f>IF(SUM(B10:B15)=0,0,SUMPRODUCT(B10:B15,G10:G15)/SUM(B10:B15))</f>
         <v/>
       </c>
     </row>
@@ -1106,7 +1154,7 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
-  <conditionalFormatting sqref="G10:G17">
+  <conditionalFormatting sqref="G10:G18">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1128,7 +1176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1154,449 +1202,513 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="40" t="inlineStr">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B4" s="40" t="inlineStr">
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="C4" s="40" t="inlineStr">
+      <c r="C4" s="43" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="D4" s="40" t="inlineStr">
+      <c r="D4" s="43" t="inlineStr">
         <is>
           <t>Days (weekdays)</t>
         </is>
       </c>
-      <c r="E4" s="40" t="inlineStr">
+      <c r="E4" s="43" t="inlineStr">
         <is>
           <t>Focus</t>
         </is>
       </c>
-      <c r="F4" s="40" t="inlineStr">
+      <c r="F4" s="43" t="inlineStr">
         <is>
           <t>Weekly Date</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="41" t="inlineStr">
+      <c r="A5" s="44" t="inlineStr">
         <is>
           <t>Phase 1 — Foundation (development)</t>
         </is>
       </c>
-      <c r="B5" s="42" t="n">
+      <c r="B5" s="45" t="n">
         <v>46224</v>
       </c>
-      <c r="C5" s="42" t="n">
+      <c r="C5" s="45" t="n">
         <v>46233</v>
       </c>
       <c r="D5" s="15">
         <f>NETWORKDAYS(B5,C5)</f>
         <v/>
       </c>
-      <c r="E5" s="41" t="inlineStr">
-        <is>
-          <t>Project setup, layout, menus, reusable UI.</t>
-        </is>
-      </c>
-      <c r="F5" s="42">
+      <c r="E5" s="44" t="inlineStr">
+        <is>
+          <t>Project setup, layout, collapsible sidebar, menus, reusable UI.</t>
+        </is>
+      </c>
+      <c r="F5" s="45">
         <f>B5+MOD(5-WEEKDAY(B5,2),7)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="43" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Phase 2 — Employee features (development)</t>
         </is>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B6" s="47" t="n">
         <v>46231</v>
       </c>
-      <c r="C6" s="44" t="n">
+      <c r="C6" s="47" t="n">
         <v>46247</v>
       </c>
       <c r="D6" s="21">
         <f>NETWORKDAYS(B6,C6)</f>
         <v/>
       </c>
-      <c r="E6" s="43" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>Dashboard, file leave, request details, history, edit, and cancel.</t>
         </is>
       </c>
-      <c r="F6" s="44">
+      <c r="F6" s="47">
         <f>B6+MOD(5-WEEKDAY(B6,2),7)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="45" t="inlineStr">
+      <c r="A7" s="48" t="inlineStr">
         <is>
           <t>Phase 3 — Approver / team (development)</t>
         </is>
       </c>
-      <c r="B7" s="46" t="n">
+      <c r="B7" s="49" t="n">
         <v>46245</v>
       </c>
-      <c r="C7" s="46" t="n">
+      <c r="C7" s="49" t="n">
         <v>46255</v>
       </c>
       <c r="D7" s="24">
         <f>NETWORKDAYS(B7,C7)</f>
         <v/>
       </c>
-      <c r="E7" s="45" t="inlineStr">
+      <c r="E7" s="48" t="inlineStr">
         <is>
           <t>Approvals inbox, approve/reject, file for member, team calendar.</t>
         </is>
       </c>
-      <c r="F7" s="46">
+      <c r="F7" s="49">
         <f>B7+MOD(5-WEEKDAY(B7,2),7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="47" t="inlineStr">
+      <c r="A8" s="50" t="inlineStr">
         <is>
           <t>Phase 4 — Admin features (development)</t>
         </is>
       </c>
-      <c r="B8" s="48" t="n">
+      <c r="B8" s="51" t="n">
         <v>46252</v>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="51" t="n">
         <v>46262</v>
       </c>
       <c r="D8" s="27">
         <f>NETWORKDAYS(B8,C8)</f>
         <v/>
       </c>
-      <c r="E8" s="47" t="inlineStr">
-        <is>
-          <t>Admin requests, conversion review, balances, logs, and reports.</t>
-        </is>
-      </c>
-      <c r="F8" s="48">
+      <c r="E8" s="50" t="inlineStr">
+        <is>
+          <t>Admin requests, conversion review, balances, logs, and all three reports (UI complete ahead of schedule).</t>
+        </is>
+      </c>
+      <c r="F8" s="51">
         <f>B8+MOD(5-WEEKDAY(B8,2),7)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="49" t="inlineStr">
-        <is>
-          <t>Phase 5 — Development complete (commitment)</t>
-        </is>
-      </c>
-      <c r="B9" s="50" t="n">
-        <v>46262</v>
-      </c>
-      <c r="C9" s="50" t="n">
-        <v>46265</v>
+      <c r="A9" s="52" t="inlineStr">
+        <is>
+          <t>Phase 5 — UI polish &amp; cleanup (development)</t>
+        </is>
+      </c>
+      <c r="B9" s="53" t="n">
+        <v>46233</v>
+      </c>
+      <c r="C9" s="53" t="n">
+        <v>46249</v>
       </c>
       <c r="D9" s="18">
         <f>NETWORKDAYS(B9,C9)</f>
         <v/>
       </c>
-      <c r="E9" s="49" t="inlineStr">
+      <c r="E9" s="52" t="inlineStr">
+        <is>
+          <t>CSS review, layout checks, and consistent spacing across screens.</t>
+        </is>
+      </c>
+      <c r="F9" s="53">
+        <f>B9+MOD(5-WEEKDAY(B9,2),7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>Phase 6 — Development complete (commitment)</t>
+        </is>
+      </c>
+      <c r="B10" s="45" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C10" s="45" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D10" s="15">
+        <f>NETWORKDAYS(B10,C10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="44" t="inlineStr">
         <is>
           <t>Frontend development screens targeted complete. End of August = development only.</t>
         </is>
       </c>
-      <c r="F9" s="50">
-        <f>B9+MOD(5-WEEKDAY(B9,2),7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="51" t="inlineStr">
+      <c r="F10" s="45">
+        <f>B10+MOD(5-WEEKDAY(B10,2),7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="54" t="inlineStr">
         <is>
           <t>After / alongside development (no fixed end dates yet)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="52" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B13" s="52" t="inlineStr">
+      <c r="B14" s="55" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="53" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="56" t="inlineStr">
         <is>
           <t>Backend integration (parallel / TBD)</t>
         </is>
       </c>
-      <c r="B14" s="53" t="inlineStr">
+      <c r="B15" s="56" t="inlineStr">
         <is>
           <t>Ongoing with backend partner — no fixed day count yet. Update when APIs and cookie/session are ready.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="54" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="57" t="inlineStr">
         <is>
           <t>Testing (after development)</t>
         </is>
       </c>
-      <c r="B15" s="54" t="inlineStr">
+      <c r="B16" s="57" t="inlineStr">
         <is>
           <t>Planned to start on/after 2026-09-01. End date TBD.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="55" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="58" t="inlineStr">
         <is>
           <t>Documentation (after development)</t>
         </is>
       </c>
-      <c r="B16" s="55" t="inlineStr">
+      <c r="B17" s="58" t="inlineStr">
         <is>
           <t>Planned to start on/after 2026-09-01. End date TBD.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="51" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="54" t="inlineStr">
         <is>
           <t>Key milestones (development)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="52" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="55" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="B20" s="52" t="inlineStr">
+      <c r="B21" s="55" t="inlineStr">
         <is>
           <t>Target Date</t>
         </is>
       </c>
-      <c r="C20" s="52" t="inlineStr">
+      <c r="C21" s="55" t="inlineStr">
         <is>
           <t>Weekly Date</t>
         </is>
       </c>
-      <c r="D20" s="52" t="inlineStr">
+      <c r="D21" s="55" t="inlineStr">
         <is>
           <t>Related section</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="56" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="59" t="inlineStr">
         <is>
           <t>App shell &amp; menus ready (dev kickoff)</t>
         </is>
       </c>
-      <c r="B21" s="57" t="n">
+      <c r="B22" s="60" t="n">
         <v>46225</v>
       </c>
-      <c r="C21" s="57">
-        <f>B21+MOD(5-WEEKDAY(B21,2),7)</f>
-        <v/>
-      </c>
-      <c r="D21" s="56" t="inlineStr">
+      <c r="C22" s="60">
+        <f>B22+MOD(5-WEEKDAY(B22,2),7)</f>
+        <v/>
+      </c>
+      <c r="D22" s="59" t="inlineStr">
         <is>
           <t>2. Core App Shell</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="56" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="59" t="inlineStr">
         <is>
           <t>Reusable UI + employee screens underway</t>
         </is>
       </c>
-      <c r="B22" s="57" t="n">
+      <c r="B23" s="60" t="n">
         <v>46234</v>
       </c>
-      <c r="C22" s="57">
-        <f>B22+MOD(5-WEEKDAY(B22,2),7)</f>
-        <v/>
-      </c>
-      <c r="D22" s="56" t="inlineStr">
+      <c r="C23" s="60">
+        <f>B23+MOD(5-WEEKDAY(B23,2),7)</f>
+        <v/>
+      </c>
+      <c r="D23" s="59" t="inlineStr">
         <is>
           <t>2–3</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="56" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="59" t="inlineStr">
         <is>
           <t>Employee filing &amp; history usable (UI)</t>
         </is>
       </c>
-      <c r="B23" s="57" t="n">
+      <c r="B24" s="60" t="n">
         <v>46247</v>
       </c>
-      <c r="C23" s="57">
-        <f>B23+MOD(5-WEEKDAY(B23,2),7)</f>
-        <v/>
-      </c>
-      <c r="D23" s="56" t="inlineStr">
+      <c r="C24" s="60">
+        <f>B24+MOD(5-WEEKDAY(B24,2),7)</f>
+        <v/>
+      </c>
+      <c r="D24" s="59" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="56" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="59" t="inlineStr">
         <is>
           <t>Approver approve/reject usable (UI)</t>
         </is>
       </c>
-      <c r="B24" s="57" t="n">
+      <c r="B25" s="60" t="n">
         <v>46252</v>
       </c>
-      <c r="C24" s="57">
-        <f>B24+MOD(5-WEEKDAY(B24,2),7)</f>
-        <v/>
-      </c>
-      <c r="D24" s="56" t="inlineStr">
+      <c r="C25" s="60">
+        <f>B25+MOD(5-WEEKDAY(B25,2),7)</f>
+        <v/>
+      </c>
+      <c r="D25" s="59" t="inlineStr">
         <is>
           <t>4. Approver / Team</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="56" t="inlineStr">
-        <is>
-          <t>Admin screens usable (UI)</t>
-        </is>
-      </c>
-      <c r="B25" s="57" t="n">
+    <row r="26">
+      <c r="A26" s="59" t="inlineStr">
+        <is>
+          <t>Admin screens usable (UI) — done early</t>
+        </is>
+      </c>
+      <c r="B26" s="60" t="n">
+        <v>46233</v>
+      </c>
+      <c r="C26" s="60">
+        <f>B26+MOD(5-WEEKDAY(B26,2),7)</f>
+        <v/>
+      </c>
+      <c r="D26" s="59" t="inlineStr">
+        <is>
+          <t>5. Admin Features</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="59" t="inlineStr">
+        <is>
+          <t>Admin screens target (original plan)</t>
+        </is>
+      </c>
+      <c r="B27" s="60" t="n">
         <v>46262</v>
       </c>
-      <c r="C25" s="57">
-        <f>B25+MOD(5-WEEKDAY(B25,2),7)</f>
-        <v/>
-      </c>
-      <c r="D25" s="56" t="inlineStr">
+      <c r="C27" s="60">
+        <f>B27+MOD(5-WEEKDAY(B27,2),7)</f>
+        <v/>
+      </c>
+      <c r="D27" s="59" t="inlineStr">
         <is>
           <t>5. Admin Features</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="56" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="59" t="inlineStr">
+        <is>
+          <t>UI polish &amp; layout cleanup underway</t>
+        </is>
+      </c>
+      <c r="B28" s="60" t="n">
+        <v>46233</v>
+      </c>
+      <c r="C28" s="60">
+        <f>B28+MOD(5-WEEKDAY(B28,2),7)</f>
+        <v/>
+      </c>
+      <c r="D28" s="59" t="inlineStr">
+        <is>
+          <t>6. UI Polish &amp; Cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="59" t="inlineStr">
         <is>
           <t>Development complete (August commitment)</t>
         </is>
       </c>
-      <c r="B26" s="57" t="n">
+      <c r="B29" s="60" t="n">
         <v>46265</v>
       </c>
-      <c r="C26" s="57">
-        <f>B26+MOD(5-WEEKDAY(B26,2),7)</f>
-        <v/>
-      </c>
-      <c r="D26" s="56" t="inlineStr">
-        <is>
-          <t>Sections 1–5</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="51" t="inlineStr">
+      <c r="C29" s="60">
+        <f>B29+MOD(5-WEEKDAY(B29,2),7)</f>
+        <v/>
+      </c>
+      <c r="D29" s="59" t="inlineStr">
+        <is>
+          <t>Sections 1–6</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="54" t="inlineStr">
         <is>
           <t>Weekly checkpoints (Fridays) — development</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="52" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="55" t="inlineStr">
         <is>
           <t>Week ending (Friday)</t>
         </is>
       </c>
-      <c r="B30" s="52" t="inlineStr">
+      <c r="B33" s="55" t="inlineStr">
         <is>
           <t>What leaders should expect to see</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="57" t="n">
+    <row r="34">
+      <c r="A34" s="60" t="n">
         <v>46227</v>
       </c>
-      <c r="B31" s="56" t="inlineStr">
+      <c r="B34" s="59" t="inlineStr">
         <is>
           <t>Kickoff: layout/menus; align cookie/session &amp; API approach with backend</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="57" t="n">
+    <row r="35">
+      <c r="A35" s="60" t="n">
         <v>46234</v>
       </c>
-      <c r="B32" s="56" t="inlineStr">
-        <is>
-          <t>Reusable UI started; employee screens beginning</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="57" t="n">
+      <c r="B35" s="59" t="inlineStr">
+        <is>
+          <t>Reusable UI done; employee + approver + admin screens largely complete (ahead of plan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="60" t="n">
         <v>46241</v>
       </c>
-      <c r="B33" s="56" t="inlineStr">
-        <is>
-          <t>Employee dashboard and file-leave UI in progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="57" t="n">
+      <c r="B36" s="59" t="inlineStr">
+        <is>
+          <t>CSS and layout cleanup in progress across screens</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="60" t="n">
         <v>46248</v>
       </c>
-      <c r="B34" s="56" t="inlineStr">
-        <is>
-          <t>Employee UI largely complete; approver screens started</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="57" t="n">
+      <c r="B37" s="59" t="inlineStr">
+        <is>
+          <t>Layout polish wrapping up; ready for backend hookup when APIs are available</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="60" t="n">
         <v>46255</v>
       </c>
-      <c r="B35" s="56" t="inlineStr">
+      <c r="B38" s="59" t="inlineStr">
         <is>
           <t>Approver UI in place; admin screens underway</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="57" t="n">
+    <row r="39">
+      <c r="A39" s="60" t="n">
         <v>46262</v>
       </c>
-      <c r="B36" s="56" t="inlineStr">
+      <c r="B39" s="59" t="inlineStr">
         <is>
           <t>Admin UI in progress / wrapping up</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="57" t="n">
+    <row r="40">
+      <c r="A40" s="60" t="n">
         <v>46265</v>
       </c>
-      <c r="B37" s="56" t="inlineStr">
+      <c r="B40" s="59" t="inlineStr">
         <is>
           <t>Target: frontend DEVELOPMENT complete (not testing/docs)</t>
         </is>
@@ -1617,7 +1729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1632,74 +1744,74 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B1" s="58" t="inlineStr">
+      <c r="B1" s="61" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" s="58" t="inlineStr">
+      <c r="C1" s="61" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="D1" s="58" t="inlineStr">
+      <c r="D1" s="61" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="E1" s="58" t="inlineStr">
+      <c r="E1" s="61" t="inlineStr">
         <is>
           <t>Days (weekdays)</t>
         </is>
       </c>
-      <c r="F1" s="58" t="inlineStr">
+      <c r="F1" s="61" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="58" t="inlineStr">
+      <c r="G1" s="61" t="inlineStr">
         <is>
           <t>Progress %</t>
         </is>
       </c>
-      <c r="H1" s="58" t="inlineStr">
+      <c r="H1" s="61" t="inlineStr">
         <is>
           <t>Weekly Date</t>
         </is>
       </c>
-      <c r="I1" s="58" t="inlineStr">
+      <c r="I1" s="61" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="41" t="inlineStr">
+      <c r="A2" s="44" t="inlineStr">
         <is>
           <t>1. Project Setup</t>
         </is>
       </c>
-      <c r="B2" s="41" t="inlineStr">
+      <c r="B2" s="44" t="inlineStr">
         <is>
           <t>Set up frontend project (React, TypeScript, styling tools)</t>
         </is>
       </c>
-      <c r="C2" s="42" t="n">
+      <c r="C2" s="45" t="n">
         <v>46224</v>
       </c>
-      <c r="D2" s="42" t="n">
+      <c r="D2" s="45" t="n">
         <v>46224</v>
       </c>
       <c r="E2" s="15">
         <f>IF(OR(C2="",D2=""),"",NETWORKDAYS(C2,D2))</f>
         <v/>
       </c>
-      <c r="F2" s="33" t="inlineStr">
+      <c r="F2" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -1708,34 +1820,34 @@
         <f>IF(F2="Completed",1,IF(F2="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H2" s="59">
+      <c r="H2" s="62">
         <f>IF(C2="","",C2+MOD(5-WEEKDAY(C2,2),7))</f>
         <v/>
       </c>
-      <c r="I2" s="41" t="inlineStr"/>
+      <c r="I2" s="44" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="41" t="inlineStr">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>1. Project Setup</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="44" t="inlineStr">
         <is>
           <t>Apply brand colors, fonts, and base page styles</t>
         </is>
       </c>
-      <c r="C3" s="42" t="n">
+      <c r="C3" s="45" t="n">
         <v>46224</v>
       </c>
-      <c r="D3" s="42" t="n">
+      <c r="D3" s="45" t="n">
         <v>46225</v>
       </c>
       <c r="E3" s="15">
         <f>IF(OR(C3="",D3=""),"",NETWORKDAYS(C3,D3))</f>
         <v/>
       </c>
-      <c r="F3" s="33" t="inlineStr">
+      <c r="F3" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -1744,34 +1856,34 @@
         <f>IF(F3="Completed",1,IF(F3="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H3" s="59">
+      <c r="H3" s="62">
         <f>IF(C3="","",C3+MOD(5-WEEKDAY(C3,2),7))</f>
         <v/>
       </c>
-      <c r="I3" s="41" t="inlineStr"/>
+      <c r="I3" s="44" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="41" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>1. Project Setup</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="44" t="inlineStr">
         <is>
           <t>Define page routes for Employee, Approver, and Admin areas</t>
         </is>
       </c>
-      <c r="C4" s="42" t="n">
+      <c r="C4" s="45" t="n">
         <v>46224</v>
       </c>
-      <c r="D4" s="42" t="n">
+      <c r="D4" s="45" t="n">
         <v>46225</v>
       </c>
       <c r="E4" s="15">
         <f>IF(OR(C4="",D4=""),"",NETWORKDAYS(C4,D4))</f>
         <v/>
       </c>
-      <c r="F4" s="33" t="inlineStr">
+      <c r="F4" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -1780,34 +1892,34 @@
         <f>IF(F4="Completed",1,IF(F4="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H4" s="59">
+      <c r="H4" s="62">
         <f>IF(C4="","",C4+MOD(5-WEEKDAY(C4,2),7))</f>
         <v/>
       </c>
-      <c r="I4" s="41" t="inlineStr"/>
+      <c r="I4" s="44" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="49" t="inlineStr">
+      <c r="A5" s="52" t="inlineStr">
         <is>
           <t>2. Core App Shell</t>
         </is>
       </c>
-      <c r="B5" s="49" t="inlineStr">
+      <c r="B5" s="52" t="inlineStr">
         <is>
           <t>Build main app layout (sidebar menu and top header)</t>
         </is>
       </c>
-      <c r="C5" s="50" t="n">
+      <c r="C5" s="53" t="n">
         <v>46224</v>
       </c>
-      <c r="D5" s="50" t="n">
+      <c r="D5" s="53" t="n">
         <v>46225</v>
       </c>
       <c r="E5" s="18">
         <f>IF(OR(C5="",D5=""),"",NETWORKDAYS(C5,D5))</f>
         <v/>
       </c>
-      <c r="F5" s="33" t="inlineStr">
+      <c r="F5" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -1816,34 +1928,34 @@
         <f>IF(F5="Completed",1,IF(F5="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H5" s="60">
+      <c r="H5" s="63">
         <f>IF(C5="","",C5+MOD(5-WEEKDAY(C5,2),7))</f>
         <v/>
       </c>
-      <c r="I5" s="49" t="inlineStr"/>
+      <c r="I5" s="52" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="49" t="inlineStr">
+      <c r="A6" s="52" t="inlineStr">
         <is>
           <t>2. Core App Shell</t>
         </is>
       </c>
-      <c r="B6" s="49" t="inlineStr">
+      <c r="B6" s="52" t="inlineStr">
         <is>
           <t>Show different menus based on user role (Employee / Approver / Admin)</t>
         </is>
       </c>
-      <c r="C6" s="50" t="n">
+      <c r="C6" s="53" t="n">
         <v>46224</v>
       </c>
-      <c r="D6" s="50" t="n">
+      <c r="D6" s="53" t="n">
         <v>46225</v>
       </c>
       <c r="E6" s="18">
         <f>IF(OR(C6="",D6=""),"",NETWORKDAYS(C6,D6))</f>
         <v/>
       </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="F6" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -1852,38 +1964,38 @@
         <f>IF(F6="Completed",1,IF(F6="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H6" s="60">
+      <c r="H6" s="63">
         <f>IF(C6="","",C6+MOD(5-WEEKDAY(C6,2),7))</f>
         <v/>
       </c>
-      <c r="I6" s="49" t="inlineStr">
+      <c r="I6" s="52" t="inlineStr">
         <is>
           <t>Role-based sidebar works. Dev-only role preview remains until portal cookies/session are wired.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="49" t="inlineStr">
+      <c r="A7" s="52" t="inlineStr">
         <is>
           <t>2. Core App Shell</t>
         </is>
       </c>
-      <c r="B7" s="49" t="inlineStr">
+      <c r="B7" s="52" t="inlineStr">
         <is>
           <t>Create reusable screen parts (buttons, forms, tables, status labels)</t>
         </is>
       </c>
-      <c r="C7" s="50" t="n">
+      <c r="C7" s="53" t="n">
         <v>46225</v>
       </c>
-      <c r="D7" s="50" t="n">
-        <v>46232</v>
+      <c r="D7" s="53" t="n">
+        <v>46233</v>
       </c>
       <c r="E7" s="18">
         <f>IF(OR(C7="",D7=""),"",NETWORKDAYS(C7,D7))</f>
         <v/>
       </c>
-      <c r="F7" s="33" t="inlineStr">
+      <c r="F7" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -1892,38 +2004,38 @@
         <f>IF(F7="Completed",1,IF(F7="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H7" s="60">
+      <c r="H7" s="63">
         <f>IF(C7="","",C7+MOD(5-WEEKDAY(C7,2),7))</f>
         <v/>
       </c>
-      <c r="I7" s="49" t="inlineStr">
-        <is>
-          <t>Built: StatusBadge, FilterSelect, Pagination, Button, Modal, ConfirmReasonModal, AttachmentPreviewModal, SuccessDialog, Skeleton, form fields, MonthYearPickerField, EmployeeMultiSelect, tableStyles, admin-specific components.</t>
+      <c r="I7" s="52" t="inlineStr">
+        <is>
+          <t>Built: StatusBadge, FilterSelect, Pagination, Button, Modal, ConfirmReasonModal, AttachmentPreviewModal, SuccessDialog, Skeleton, form fields, MonthYearPickerField, YearPickerField, EmployeeMultiSelect, tableStyles, admin-specific components.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="49" t="inlineStr">
+      <c r="A8" s="52" t="inlineStr">
         <is>
           <t>2. Core App Shell</t>
         </is>
       </c>
-      <c r="B8" s="49" t="inlineStr">
-        <is>
-          <t>Replace temporary placeholder pages with real screens</t>
-        </is>
-      </c>
-      <c r="C8" s="50" t="n">
-        <v>46225</v>
-      </c>
-      <c r="D8" s="50" t="n">
+      <c r="B8" s="52" t="inlineStr">
+        <is>
+          <t>Collapsible sidebar menu with saved user preference</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="n">
         <v>46232</v>
+      </c>
+      <c r="D8" s="53" t="n">
+        <v>46233</v>
       </c>
       <c r="E8" s="18">
         <f>IF(OR(C8="",D8=""),"",NETWORKDAYS(C8,D8))</f>
         <v/>
       </c>
-      <c r="F8" s="33" t="inlineStr">
+      <c r="F8" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -1932,78 +2044,78 @@
         <f>IF(F8="Completed",1,IF(F8="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H8" s="60">
+      <c r="H8" s="63">
         <f>IF(C8="","",C8+MOD(5-WEEKDAY(C8,2),7))</f>
         <v/>
       </c>
-      <c r="I8" s="49" t="inlineStr">
-        <is>
-          <t>All employee, approver/team, and admin routes now have real page components. No PagePlaceholder routes remain (only 2 minor sub-reports still placeholders).</t>
+      <c r="I8" s="52" t="inlineStr">
+        <is>
+          <t>Sidebar collapses to icon-only mode with flyout submenus, tooltips, and localStorage preference. Top header toggle wired in AppLayout.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="43" t="inlineStr">
+      <c r="A9" s="52" t="inlineStr">
+        <is>
+          <t>2. Core App Shell</t>
+        </is>
+      </c>
+      <c r="B9" s="52" t="inlineStr">
+        <is>
+          <t>Replace temporary placeholder pages with real screens</t>
+        </is>
+      </c>
+      <c r="C9" s="53" t="n">
+        <v>46225</v>
+      </c>
+      <c r="D9" s="53" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E9" s="18">
+        <f>IF(OR(C9="",D9=""),"",NETWORKDAYS(C9,D9))</f>
+        <v/>
+      </c>
+      <c r="F9" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G9" s="19">
+        <f>IF(F9="Completed",1,IF(F9="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H9" s="63">
+        <f>IF(C9="","",C9+MOD(5-WEEKDAY(C9,2),7))</f>
+        <v/>
+      </c>
+      <c r="I9" s="52" t="inlineStr">
+        <is>
+          <t>All employee, approver/team, and admin routes now have real page components. PagePlaceholder is no longer used in routing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="46" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
-      <c r="B9" s="43" t="inlineStr">
+      <c r="B10" s="46" t="inlineStr">
         <is>
           <t>Employee dashboard: leave balances and recent requests</t>
         </is>
       </c>
-      <c r="C9" s="44" t="n">
+      <c r="C10" s="47" t="n">
         <v>46225</v>
       </c>
-      <c r="D9" s="44" t="n">
+      <c r="D10" s="47" t="n">
         <v>46225</v>
-      </c>
-      <c r="E9" s="21">
-        <f>IF(OR(C9="",D9=""),"",NETWORKDAYS(C9,D9))</f>
-        <v/>
-      </c>
-      <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="G9" s="22">
-        <f>IF(F9="Completed",1,IF(F9="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H9" s="61">
-        <f>IF(C9="","",C9+MOD(5-WEEKDAY(C9,2),7))</f>
-        <v/>
-      </c>
-      <c r="I9" s="43" t="inlineStr">
-        <is>
-          <t>UI complete (balances, reserved credits, filters, pagination). Uses mock data until Backend Integration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="43" t="inlineStr">
-        <is>
-          <t>3. Employee Features</t>
-        </is>
-      </c>
-      <c r="B10" s="43" t="inlineStr">
-        <is>
-          <t>File leave request (dates, leave type, reason, attachment)</t>
-        </is>
-      </c>
-      <c r="C10" s="44" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D10" s="44" t="n">
-        <v>46226</v>
       </c>
       <c r="E10" s="21">
         <f>IF(OR(C10="",D10=""),"",NETWORKDAYS(C10,D10))</f>
         <v/>
       </c>
-      <c r="F10" s="33" t="inlineStr">
+      <c r="F10" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2012,38 +2124,38 @@
         <f>IF(F10="Completed",1,IF(F10="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H10" s="61">
+      <c r="H10" s="64">
         <f>IF(C10="","",C10+MOD(5-WEEKDAY(C10,2),7))</f>
         <v/>
       </c>
-      <c r="I10" s="43" t="inlineStr">
-        <is>
-          <t>Apply Leave page is built with employee info, leave type/day type, date range, reason, attachment rules, duration preview, confirm modal, and success dialog. Uses mock submit until Backend Integration.</t>
+      <c r="I10" s="46" t="inlineStr">
+        <is>
+          <t>UI complete (balances, reserved credits, filters, pagination). Uses mock data until Backend Integration.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="46" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
-        <is>
-          <t>Show unpaid leave (LWOP) warning when credits are not enough</t>
-        </is>
-      </c>
-      <c r="C11" s="44" t="n">
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>File leave request (dates, leave type, reason, attachment)</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="n">
         <v>46226</v>
       </c>
-      <c r="D11" s="44" t="n">
+      <c r="D11" s="47" t="n">
         <v>46226</v>
       </c>
       <c r="E11" s="21">
         <f>IF(OR(C11="",D11=""),"",NETWORKDAYS(C11,D11))</f>
         <v/>
       </c>
-      <c r="F11" s="33" t="inlineStr">
+      <c r="F11" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2052,38 +2164,38 @@
         <f>IF(F11="Completed",1,IF(F11="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H11" s="61">
+      <c r="H11" s="64">
         <f>IF(C11="","",C11+MOD(5-WEEKDAY(C11,2),7))</f>
         <v/>
       </c>
-      <c r="I11" s="43" t="inlineStr">
-        <is>
-          <t>LWOP / remaining-balance warning is shown in filing forms using mock remaining-day logic.</t>
+      <c r="I11" s="46" t="inlineStr">
+        <is>
+          <t>Apply Leave page is built with employee info, leave type/day type, date range, reason, attachment rules, duration preview, confirm modal, and success dialog. Uses mock submit until Backend Integration.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="43" t="inlineStr">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
-      <c r="B12" s="43" t="inlineStr">
-        <is>
-          <t>Leave request details: status, approvals needed, and activity history</t>
-        </is>
-      </c>
-      <c r="C12" s="44" t="n">
-        <v>46225</v>
-      </c>
-      <c r="D12" s="44" t="n">
-        <v>46225</v>
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>Show unpaid leave (LWOP) warning when credits are not enough</t>
+        </is>
+      </c>
+      <c r="C12" s="47" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D12" s="47" t="n">
+        <v>46226</v>
       </c>
       <c r="E12" s="21">
         <f>IF(OR(C12="",D12=""),"",NETWORKDAYS(C12,D12))</f>
         <v/>
       </c>
-      <c r="F12" s="33" t="inlineStr">
+      <c r="F12" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2092,38 +2204,38 @@
         <f>IF(F12="Completed",1,IF(F12="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H12" s="61">
+      <c r="H12" s="64">
         <f>IF(C12="","",C12+MOD(5-WEEKDAY(C12,2),7))</f>
         <v/>
       </c>
-      <c r="I12" s="43" t="inlineStr">
-        <is>
-          <t>UI complete: leave info, approval progress/requirements, approver list, attachments, conversion view. Mock data; activity timeline not a separate log yet.</t>
+      <c r="I12" s="46" t="inlineStr">
+        <is>
+          <t>LWOP / remaining-balance warning is shown in filing forms using mock remaining-day logic.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="A13" s="46" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
-        <is>
-          <t>Activity log / leave history with filters</t>
-        </is>
-      </c>
-      <c r="C13" s="44" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D13" s="44" t="n">
-        <v>46226</v>
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t>Leave request details: status, approvals needed, and activity history</t>
+        </is>
+      </c>
+      <c r="C13" s="47" t="n">
+        <v>46225</v>
+      </c>
+      <c r="D13" s="47" t="n">
+        <v>46225</v>
       </c>
       <c r="E13" s="21">
         <f>IF(OR(C13="",D13=""),"",NETWORKDAYS(C13,D13))</f>
         <v/>
       </c>
-      <c r="F13" s="33" t="inlineStr">
+      <c r="F13" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2132,38 +2244,38 @@
         <f>IF(F13="Completed",1,IF(F13="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H13" s="61">
+      <c r="H13" s="64">
         <f>IF(C13="","",C13+MOD(5-WEEKDAY(C13,2),7))</f>
         <v/>
       </c>
-      <c r="I13" s="43" t="inlineStr">
-        <is>
-          <t>Activity Log page exists with filtering, sorting, pagination, and mock activity data.</t>
+      <c r="I13" s="46" t="inlineStr">
+        <is>
+          <t>UI complete: leave info, approval progress/requirements, approver list, attachments, conversion view. Mock data; activity timeline not a separate log yet.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="43" t="inlineStr">
+      <c r="A14" s="46" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
-      <c r="B14" s="43" t="inlineStr">
-        <is>
-          <t>Edit leave request (only while still waiting for first approval)</t>
-        </is>
-      </c>
-      <c r="C14" s="44" t="n">
-        <v>46225</v>
-      </c>
-      <c r="D14" s="44" t="n">
-        <v>46247</v>
+      <c r="B14" s="46" t="inlineStr">
+        <is>
+          <t>Activity log / leave history with filters</t>
+        </is>
+      </c>
+      <c r="C14" s="47" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D14" s="47" t="n">
+        <v>46226</v>
       </c>
       <c r="E14" s="21">
         <f>IF(OR(C14="",D14=""),"",NETWORKDAYS(C14,D14))</f>
         <v/>
       </c>
-      <c r="F14" s="33" t="inlineStr">
+      <c r="F14" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2172,38 +2284,38 @@
         <f>IF(F14="Completed",1,IF(F14="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H14" s="61">
+      <c r="H14" s="64">
         <f>IF(C14="","",C14+MOD(5-WEEKDAY(C14,2),7))</f>
         <v/>
       </c>
-      <c r="I14" s="43" t="inlineStr">
-        <is>
-          <t>Edit Leave page exists with date/day-type/reason editing, weekday duration recalculation, lead-time validation, confirm modal, and rules from details page. Uses mock save until Backend Integration.</t>
+      <c r="I14" s="46" t="inlineStr">
+        <is>
+          <t>Activity Log page exists with filtering, sorting, pagination, and mock activity data.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="43" t="inlineStr">
+      <c r="A15" s="46" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
-      <c r="B15" s="43" t="inlineStr">
-        <is>
-          <t>Cancel leave request (with required reason)</t>
-        </is>
-      </c>
-      <c r="C15" s="44" t="n">
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>Edit leave request (only while still waiting for first approval)</t>
+        </is>
+      </c>
+      <c r="C15" s="47" t="n">
         <v>46225</v>
       </c>
-      <c r="D15" s="44" t="n">
+      <c r="D15" s="47" t="n">
         <v>46247</v>
       </c>
       <c r="E15" s="21">
         <f>IF(OR(C15="",D15=""),"",NETWORKDAYS(C15,D15))</f>
         <v/>
       </c>
-      <c r="F15" s="33" t="inlineStr">
+      <c r="F15" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2212,38 +2324,38 @@
         <f>IF(F15="Completed",1,IF(F15="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H15" s="61">
+      <c r="H15" s="64">
         <f>IF(C15="","",C15+MOD(5-WEEKDAY(C15,2),7))</f>
         <v/>
       </c>
-      <c r="I15" s="43" t="inlineStr">
-        <is>
-          <t>Cancel flow is present on details page with required-reason modal and success state. Uses mock action until Backend Integration.</t>
+      <c r="I15" s="46" t="inlineStr">
+        <is>
+          <t>Edit Leave page exists with date/day-type/reason editing, weekday duration recalculation, lead-time validation, confirm modal, and rules from details page. Uses mock save until Backend Integration.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="43" t="inlineStr">
+      <c r="A16" s="46" t="inlineStr">
         <is>
           <t>3. Employee Features</t>
         </is>
       </c>
-      <c r="B16" s="43" t="inlineStr">
-        <is>
-          <t>Request vacation-to-sick leave conversion (upload medical certificate)</t>
-        </is>
-      </c>
-      <c r="C16" s="44" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D16" s="44" t="n">
-        <v>46226</v>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t>Cancel leave request (with required reason)</t>
+        </is>
+      </c>
+      <c r="C16" s="47" t="n">
+        <v>46225</v>
+      </c>
+      <c r="D16" s="47" t="n">
+        <v>46247</v>
       </c>
       <c r="E16" s="21">
         <f>IF(OR(C16="",D16=""),"",NETWORKDAYS(C16,D16))</f>
         <v/>
       </c>
-      <c r="F16" s="33" t="inlineStr">
+      <c r="F16" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2252,78 +2364,78 @@
         <f>IF(F16="Completed",1,IF(F16="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H16" s="61">
+      <c r="H16" s="64">
         <f>IF(C16="","",C16+MOD(5-WEEKDAY(C16,2),7))</f>
         <v/>
       </c>
-      <c r="I16" s="43" t="inlineStr">
+      <c r="I16" s="46" t="inlineStr">
+        <is>
+          <t>Cancel flow is present on details page with required-reason modal and success state. Uses mock action until Backend Integration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="46" t="inlineStr">
+        <is>
+          <t>3. Employee Features</t>
+        </is>
+      </c>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>Request vacation-to-sick leave conversion (upload medical certificate)</t>
+        </is>
+      </c>
+      <c r="C17" s="47" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D17" s="47" t="n">
+        <v>46226</v>
+      </c>
+      <c r="E17" s="21">
+        <f>IF(OR(C17="",D17=""),"",NETWORKDAYS(C17,D17))</f>
+        <v/>
+      </c>
+      <c r="F17" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G17" s="22">
+        <f>IF(F17="Completed",1,IF(F17="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H17" s="64">
+        <f>IF(C17="","",C17+MOD(5-WEEKDAY(C17,2),7))</f>
+        <v/>
+      </c>
+      <c r="I17" s="46" t="inlineStr">
         <is>
           <t>Conversion page exists with reason + medical certificate upload, eligibility rules, confirm modal, and mock submission.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="45" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="48" t="inlineStr">
         <is>
           <t>4. Approver / Team Features</t>
         </is>
       </c>
-      <c r="B17" s="45" t="inlineStr">
+      <c r="B18" s="48" t="inlineStr">
         <is>
           <t>Approver inbox: list of leave requests waiting for action</t>
         </is>
       </c>
-      <c r="C17" s="46" t="n">
+      <c r="C18" s="49" t="n">
         <v>46226</v>
       </c>
-      <c r="D17" s="46" t="n">
-        <v>46226</v>
-      </c>
-      <c r="E17" s="24">
-        <f>IF(OR(C17="",D17=""),"",NETWORKDAYS(C17,D17))</f>
-        <v/>
-      </c>
-      <c r="F17" s="33" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="G17" s="25">
-        <f>IF(F17="Completed",1,IF(F17="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H17" s="62">
-        <f>IF(C17="","",C17+MOD(5-WEEKDAY(C17,2),7))</f>
-        <v/>
-      </c>
-      <c r="I17" s="45" t="inlineStr">
-        <is>
-          <t>Leave Approvals page exists with pending/all tabs, search, filters, sorting, pagination, and mock queue data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="45" t="inlineStr">
-        <is>
-          <t>4. Approver / Team Features</t>
-        </is>
-      </c>
-      <c r="B18" s="45" t="inlineStr">
-        <is>
-          <t>Approve or reject leave (reject requires remarks)</t>
-        </is>
-      </c>
-      <c r="C18" s="46" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D18" s="46" t="n">
+      <c r="D18" s="49" t="n">
         <v>46226</v>
       </c>
       <c r="E18" s="24">
         <f>IF(OR(C18="",D18=""),"",NETWORKDAYS(C18,D18))</f>
         <v/>
       </c>
-      <c r="F18" s="33" t="inlineStr">
+      <c r="F18" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2332,38 +2444,38 @@
         <f>IF(F18="Completed",1,IF(F18="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H18" s="62">
+      <c r="H18" s="65">
         <f>IF(C18="","",C18+MOD(5-WEEKDAY(C18,2),7))</f>
         <v/>
       </c>
-      <c r="I18" s="45" t="inlineStr">
-        <is>
-          <t>Review page supports approve/reject actions, required rejection reason, confirmation modals, and success dialogs. Uses mock actions until Backend Integration.</t>
+      <c r="I18" s="48" t="inlineStr">
+        <is>
+          <t>Leave Approvals page exists with pending/all tabs, search, filters, sorting, pagination, and mock queue data.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="45" t="inlineStr">
+      <c r="A19" s="48" t="inlineStr">
         <is>
           <t>4. Approver / Team Features</t>
         </is>
       </c>
-      <c r="B19" s="45" t="inlineStr">
-        <is>
-          <t>Show clear approval progress (who still needs to act)</t>
-        </is>
-      </c>
-      <c r="C19" s="46" t="n">
-        <v>46225</v>
-      </c>
-      <c r="D19" s="46" t="n">
-        <v>46252</v>
+      <c r="B19" s="48" t="inlineStr">
+        <is>
+          <t>Approve or reject leave (reject requires remarks)</t>
+        </is>
+      </c>
+      <c r="C19" s="49" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D19" s="49" t="n">
+        <v>46226</v>
       </c>
       <c r="E19" s="24">
         <f>IF(OR(C19="",D19=""),"",NETWORKDAYS(C19,D19))</f>
         <v/>
       </c>
-      <c r="F19" s="33" t="inlineStr">
+      <c r="F19" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2372,38 +2484,38 @@
         <f>IF(F19="Completed",1,IF(F19="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H19" s="62">
+      <c r="H19" s="65">
         <f>IF(C19="","",C19+MOD(5-WEEKDAY(C19,2),7))</f>
         <v/>
       </c>
-      <c r="I19" s="45" t="inlineStr">
-        <is>
-          <t>Approval progress bars, requirement checklist, and approver status tables are built on employee details and approver review pages.</t>
+      <c r="I19" s="48" t="inlineStr">
+        <is>
+          <t>Review page supports approve/reject actions, required rejection reason, confirmation modals, and success dialogs. Uses mock actions until Backend Integration.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="45" t="inlineStr">
+      <c r="A20" s="48" t="inlineStr">
         <is>
           <t>4. Approver / Team Features</t>
         </is>
       </c>
-      <c r="B20" s="45" t="inlineStr">
-        <is>
-          <t>File leave on behalf of a team member</t>
-        </is>
-      </c>
-      <c r="C20" s="46" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D20" s="46" t="n">
-        <v>46226</v>
+      <c r="B20" s="48" t="inlineStr">
+        <is>
+          <t>Show clear approval progress (who still needs to act)</t>
+        </is>
+      </c>
+      <c r="C20" s="49" t="n">
+        <v>46225</v>
+      </c>
+      <c r="D20" s="49" t="n">
+        <v>46252</v>
       </c>
       <c r="E20" s="24">
         <f>IF(OR(C20="",D20=""),"",NETWORKDAYS(C20,D20))</f>
         <v/>
       </c>
-      <c r="F20" s="33" t="inlineStr">
+      <c r="F20" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2412,38 +2524,38 @@
         <f>IF(F20="Completed",1,IF(F20="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H20" s="62">
+      <c r="H20" s="65">
         <f>IF(C20="","",C20+MOD(5-WEEKDAY(C20,2),7))</f>
         <v/>
       </c>
-      <c r="I20" s="45" t="inlineStr">
-        <is>
-          <t>File Leave for Member page exists with member selection, leave form, LWOP warning, attachment rules, confirm modal, and mock submit.</t>
+      <c r="I20" s="48" t="inlineStr">
+        <is>
+          <t>Approval progress bars, requirement checklist, and approver status tables are built on employee details and approver review pages.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="45" t="inlineStr">
+      <c r="A21" s="48" t="inlineStr">
         <is>
           <t>4. Approver / Team Features</t>
         </is>
       </c>
-      <c r="B21" s="45" t="inlineStr">
-        <is>
-          <t>Team leave calendar and upcoming approved leaves</t>
-        </is>
-      </c>
-      <c r="C21" s="46" t="n">
-        <v>46232</v>
-      </c>
-      <c r="D21" s="46" t="n">
-        <v>46232</v>
+      <c r="B21" s="48" t="inlineStr">
+        <is>
+          <t>File leave on behalf of a team member</t>
+        </is>
+      </c>
+      <c r="C21" s="49" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D21" s="49" t="n">
+        <v>46226</v>
       </c>
       <c r="E21" s="24">
         <f>IF(OR(C21="",D21=""),"",NETWORKDAYS(C21,D21))</f>
         <v/>
       </c>
-      <c r="F21" s="33" t="inlineStr">
+      <c r="F21" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2452,78 +2564,78 @@
         <f>IF(F21="Completed",1,IF(F21="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H21" s="62">
+      <c r="H21" s="65">
         <f>IF(C21="","",C21+MOD(5-WEEKDAY(C21,2),7))</f>
         <v/>
       </c>
-      <c r="I21" s="45" t="inlineStr">
+      <c r="I21" s="48" t="inlineStr">
+        <is>
+          <t>File Leave for Member page exists with member selection, leave form, LWOP warning, attachment rules, confirm modal, and mock submit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="48" t="inlineStr">
+        <is>
+          <t>4. Approver / Team Features</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="inlineStr">
+        <is>
+          <t>Team leave calendar and upcoming approved leaves</t>
+        </is>
+      </c>
+      <c r="C22" s="49" t="n">
+        <v>46232</v>
+      </c>
+      <c r="D22" s="49" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E22" s="24">
+        <f>IF(OR(C22="",D22=""),"",NETWORKDAYS(C22,D22))</f>
+        <v/>
+      </c>
+      <c r="F22" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G22" s="25">
+        <f>IF(F22="Completed",1,IF(F22="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H22" s="65">
+        <f>IF(C22="","",C22+MOD(5-WEEKDAY(C22,2),7))</f>
+        <v/>
+      </c>
+      <c r="I22" s="48" t="inlineStr">
         <is>
           <t>Team Leave Calendar page (month/week views, filters, leave chips) and Upcoming Approved Leaves page are both built with mock data.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="47" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="50" t="inlineStr">
         <is>
           <t>5. Admin Features</t>
         </is>
       </c>
-      <c r="B22" s="47" t="inlineStr">
+      <c r="B23" s="50" t="inlineStr">
         <is>
           <t>Admin view of leave requests and request details</t>
         </is>
       </c>
-      <c r="C22" s="48" t="n">
+      <c r="C23" s="51" t="n">
         <v>46232</v>
       </c>
-      <c r="D22" s="48" t="n">
-        <v>46232</v>
-      </c>
-      <c r="E22" s="27">
-        <f>IF(OR(C22="",D22=""),"",NETWORKDAYS(C22,D22))</f>
-        <v/>
-      </c>
-      <c r="F22" s="33" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="G22" s="28">
-        <f>IF(F22="Completed",1,IF(F22="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H22" s="63">
-        <f>IF(C22="","",C22+MOD(5-WEEKDAY(C22,2),7))</f>
-        <v/>
-      </c>
-      <c r="I22" s="47" t="inlineStr">
-        <is>
-          <t>Admin Leave Requests list (pending/all tabs, filters, search, reminders) and detail/view/validate pages are all built with mock data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="47" t="inlineStr">
-        <is>
-          <t>5. Admin Features</t>
-        </is>
-      </c>
-      <c r="B23" s="47" t="inlineStr">
-        <is>
-          <t>Review vacation-to-sick leave conversion requests</t>
-        </is>
-      </c>
-      <c r="C23" s="48" t="n">
-        <v>46232</v>
-      </c>
-      <c r="D23" s="48" t="n">
+      <c r="D23" s="51" t="n">
         <v>46232</v>
       </c>
       <c r="E23" s="27">
         <f>IF(OR(C23="",D23=""),"",NETWORKDAYS(C23,D23))</f>
         <v/>
       </c>
-      <c r="F23" s="33" t="inlineStr">
+      <c r="F23" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2532,38 +2644,38 @@
         <f>IF(F23="Completed",1,IF(F23="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H23" s="63">
+      <c r="H23" s="66">
         <f>IF(C23="","",C23+MOD(5-WEEKDAY(C23,2),7))</f>
         <v/>
       </c>
-      <c r="I23" s="47" t="inlineStr">
-        <is>
-          <t>Conversion review is handled via Admin Leave Validate page; conversion state visible on request detail/view pages.</t>
+      <c r="I23" s="50" t="inlineStr">
+        <is>
+          <t>Admin Leave Requests list (pending/all tabs, filters, search, reminders) and detail/view/validate pages are all built with mock data.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="47" t="inlineStr">
+      <c r="A24" s="50" t="inlineStr">
         <is>
           <t>5. Admin Features</t>
         </is>
       </c>
-      <c r="B24" s="47" t="inlineStr">
-        <is>
-          <t>Manage leave balances and credit distribution</t>
-        </is>
-      </c>
-      <c r="C24" s="48" t="n">
+      <c r="B24" s="50" t="inlineStr">
+        <is>
+          <t>Review vacation-to-sick leave conversion requests</t>
+        </is>
+      </c>
+      <c r="C24" s="51" t="n">
         <v>46232</v>
       </c>
-      <c r="D24" s="48" t="n">
+      <c r="D24" s="51" t="n">
         <v>46232</v>
       </c>
       <c r="E24" s="27">
         <f>IF(OR(C24="",D24=""),"",NETWORKDAYS(C24,D24))</f>
         <v/>
       </c>
-      <c r="F24" s="33" t="inlineStr">
+      <c r="F24" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2572,38 +2684,38 @@
         <f>IF(F24="Completed",1,IF(F24="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H24" s="63">
+      <c r="H24" s="66">
         <f>IF(C24="","",C24+MOD(5-WEEKDAY(C24,2),7))</f>
         <v/>
       </c>
-      <c r="I24" s="47" t="inlineStr">
-        <is>
-          <t>Admin Leave Balances page with filters, adjust-credits modal, and full distribution flows (annual, newly-regularized, parental, contractual) are built with mock data.</t>
+      <c r="I24" s="50" t="inlineStr">
+        <is>
+          <t>Conversion review is handled via Admin Leave Validate page; conversion state visible on request detail/view pages.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="47" t="inlineStr">
+      <c r="A25" s="50" t="inlineStr">
         <is>
           <t>5. Admin Features</t>
         </is>
       </c>
-      <c r="B25" s="47" t="inlineStr">
-        <is>
-          <t>Administrative logs</t>
-        </is>
-      </c>
-      <c r="C25" s="48" t="n">
+      <c r="B25" s="50" t="inlineStr">
+        <is>
+          <t>Manage leave balances and credit distribution</t>
+        </is>
+      </c>
+      <c r="C25" s="51" t="n">
         <v>46232</v>
       </c>
-      <c r="D25" s="48" t="n">
+      <c r="D25" s="51" t="n">
         <v>46232</v>
       </c>
       <c r="E25" s="27">
         <f>IF(OR(C25="",D25=""),"",NETWORKDAYS(C25,D25))</f>
         <v/>
       </c>
-      <c r="F25" s="33" t="inlineStr">
+      <c r="F25" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2612,78 +2724,78 @@
         <f>IF(F25="Completed",1,IF(F25="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H25" s="63">
+      <c r="H25" s="66">
         <f>IF(C25="","",C25+MOD(5-WEEKDAY(C25,2),7))</f>
         <v/>
       </c>
-      <c r="I25" s="47" t="inlineStr">
-        <is>
-          <t>Admin Administrative Log page with search, filters, month-year picker, sorting, and pagination is built with mock data.</t>
+      <c r="I25" s="50" t="inlineStr">
+        <is>
+          <t>Admin Leave Balances page with filters, adjust-credits modal, and full distribution flows (annual, newly-regularized, parental, contractual) are built with mock data.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="47" t="inlineStr">
+      <c r="A26" s="50" t="inlineStr">
         <is>
           <t>5. Admin Features</t>
         </is>
       </c>
-      <c r="B26" s="47" t="inlineStr">
-        <is>
-          <t>Leave reports for management review</t>
-        </is>
-      </c>
-      <c r="C26" s="48" t="n">
+      <c r="B26" s="50" t="inlineStr">
+        <is>
+          <t>Administrative logs</t>
+        </is>
+      </c>
+      <c r="C26" s="51" t="n">
         <v>46232</v>
       </c>
-      <c r="D26" s="48" t="n">
+      <c r="D26" s="51" t="n">
         <v>46232</v>
       </c>
       <c r="E26" s="27">
         <f>IF(OR(C26="",D26=""),"",NETWORKDAYS(C26,D26))</f>
         <v/>
       </c>
-      <c r="F26" s="64" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="F26" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G26" s="28">
         <f>IF(F26="Completed",1,IF(F26="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H26" s="63">
+      <c r="H26" s="66">
         <f>IF(C26="","",C26+MOD(5-WEEKDAY(C26,2),7))</f>
         <v/>
       </c>
-      <c r="I26" s="47" t="inlineStr">
-        <is>
-          <t>Monthly Attendance Report page built. Leave Monetization Candidates and Employees with LWOP sub-reports are still placeholders.</t>
+      <c r="I26" s="50" t="inlineStr">
+        <is>
+          <t>Admin Administrative Log page with search, filters, month-year picker, sorting, and pagination is built with mock data.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="47" t="inlineStr">
+      <c r="A27" s="50" t="inlineStr">
         <is>
           <t>5. Admin Features</t>
         </is>
       </c>
-      <c r="B27" s="47" t="inlineStr">
-        <is>
-          <t>Support other leave types (emergency, maternity, etc.) in the screens</t>
-        </is>
-      </c>
-      <c r="C27" s="48" t="n">
-        <v>46225</v>
-      </c>
-      <c r="D27" s="48" t="n">
+      <c r="B27" s="50" t="inlineStr">
+        <is>
+          <t>Monthly Attendance Report</t>
+        </is>
+      </c>
+      <c r="C27" s="51" t="n">
+        <v>46232</v>
+      </c>
+      <c r="D27" s="51" t="n">
         <v>46232</v>
       </c>
       <c r="E27" s="27">
         <f>IF(OR(C27="",D27=""),"",NETWORKDAYS(C27,D27))</f>
         <v/>
       </c>
-      <c r="F27" s="33" t="inlineStr">
+      <c r="F27" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -2692,256 +2804,276 @@
         <f>IF(F27="Completed",1,IF(F27="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H27" s="63">
+      <c r="H27" s="66">
         <f>IF(C27="","",C27+MOD(5-WEEKDAY(C27,2),7))</f>
         <v/>
       </c>
-      <c r="I27" s="47" t="inlineStr">
+      <c r="I27" s="50" t="inlineStr">
+        <is>
+          <t>Report page with month/cut-off filters, employee multi-select, group filter, calendar grid, legend, print, and download. Uses mock data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>5. Admin Features</t>
+        </is>
+      </c>
+      <c r="B28" s="50" t="inlineStr">
+        <is>
+          <t>Leave Monetization Candidates report</t>
+        </is>
+      </c>
+      <c r="C28" s="51" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D28" s="51" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E28" s="27">
+        <f>IF(OR(C28="",D28=""),"",NETWORKDAYS(C28,D28))</f>
+        <v/>
+      </c>
+      <c r="F28" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G28" s="28">
+        <f>IF(F28="Completed",1,IF(F28="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H28" s="66">
+        <f>IF(C28="","",C28+MOD(5-WEEKDAY(C28,2),7))</f>
+        <v/>
+      </c>
+      <c r="I28" s="50" t="inlineStr">
+        <is>
+          <t>Report page with year filter, eligibility filters, sortable table, summary totals, print, and download. Uses mock data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="50" t="inlineStr">
+        <is>
+          <t>5. Admin Features</t>
+        </is>
+      </c>
+      <c r="B29" s="50" t="inlineStr">
+        <is>
+          <t>Employees with LWOP report</t>
+        </is>
+      </c>
+      <c r="C29" s="51" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D29" s="51" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E29" s="27">
+        <f>IF(OR(C29="",D29=""),"",NETWORKDAYS(C29,D29))</f>
+        <v/>
+      </c>
+      <c r="F29" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G29" s="28">
+        <f>IF(F29="Completed",1,IF(F29="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H29" s="66">
+        <f>IF(C29="","",C29+MOD(5-WEEKDAY(C29,2),7))</f>
+        <v/>
+      </c>
+      <c r="I29" s="50" t="inlineStr">
+        <is>
+          <t>Report page with year and group filters, sortable LWOP summary table, print, and download. Uses mock data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="50" t="inlineStr">
+        <is>
+          <t>5. Admin Features</t>
+        </is>
+      </c>
+      <c r="B30" s="50" t="inlineStr">
+        <is>
+          <t>Support other leave types (emergency, maternity, etc.) in the screens</t>
+        </is>
+      </c>
+      <c r="C30" s="51" t="n">
+        <v>46225</v>
+      </c>
+      <c r="D30" s="51" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E30" s="27">
+        <f>IF(OR(C30="",D30=""),"",NETWORKDAYS(C30,D30))</f>
+        <v/>
+      </c>
+      <c r="F30" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G30" s="28">
+        <f>IF(F30="Completed",1,IF(F30="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H30" s="66">
+        <f>IF(C30="","",C30+MOD(5-WEEKDAY(C30,2),7))</f>
+        <v/>
+      </c>
+      <c r="I30" s="50" t="inlineStr">
         <is>
           <t>Emergency, PTB, Maternity/Paternity handled in employee/team filing and in admin screens. Monthly attendance report covers all leave categories including LWOP.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="53" t="inlineStr">
-        <is>
-          <t>6. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B28" s="53" t="inlineStr">
-        <is>
-          <t>Connect frontend to backend API (base connection and shared data types)</t>
-        </is>
-      </c>
-      <c r="C28" s="65" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D28" s="65" t="n"/>
-      <c r="E28" s="30">
-        <f>IF(OR(C28="",D28=""),"",NETWORKDAYS(C28,D28))</f>
-        <v/>
-      </c>
-      <c r="F28" s="66" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G28" s="31">
-        <f>IF(F28="Completed",1,IF(F28="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H28" s="67">
-        <f>IF(C28="","",C28+MOD(5-WEEKDAY(C28,2),7))</f>
-        <v/>
-      </c>
-      <c r="I28" s="53" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="53" t="inlineStr">
-        <is>
-          <t>6. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B29" s="53" t="inlineStr">
-        <is>
-          <t>Use portal cookies / session to identify the user (no separate login page)</t>
-        </is>
-      </c>
-      <c r="C29" s="65" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D29" s="65" t="n"/>
-      <c r="E29" s="30">
-        <f>IF(OR(C29="",D29=""),"",NETWORKDAYS(C29,D29))</f>
-        <v/>
-      </c>
-      <c r="F29" s="66" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G29" s="31">
-        <f>IF(F29="Completed",1,IF(F29="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H29" s="67">
-        <f>IF(C29="","",C29+MOD(5-WEEKDAY(C29,2),7))</f>
-        <v/>
-      </c>
-      <c r="I29" s="53" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known. Agreed with backend: cookies/session — no login screen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="53" t="inlineStr">
-        <is>
-          <t>6. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B30" s="53" t="inlineStr">
-        <is>
-          <t>Connect employee leave screens to live API (file, history, cancel, edit)</t>
-        </is>
-      </c>
-      <c r="C30" s="65" t="n"/>
-      <c r="D30" s="65" t="n"/>
-      <c r="E30" s="30">
-        <f>IF(OR(C30="",D30=""),"",NETWORKDAYS(C30,D30))</f>
-        <v/>
-      </c>
-      <c r="F30" s="66" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G30" s="31">
-        <f>IF(F30="Completed",1,IF(F30="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H30" s="67">
-        <f>IF(C30="","",C30+MOD(5-WEEKDAY(C30,2),7))</f>
-        <v/>
-      </c>
-      <c r="I30" s="53" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
-        </is>
-      </c>
-    </row>
     <row r="31">
-      <c r="A31" s="53" t="inlineStr">
-        <is>
-          <t>6. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B31" s="53" t="inlineStr">
-        <is>
-          <t>Connect approver / team screens to live API (inbox, approve, reject)</t>
-        </is>
-      </c>
-      <c r="C31" s="65" t="n"/>
-      <c r="D31" s="65" t="n"/>
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>6. UI Polish &amp; Cleanup</t>
+        </is>
+      </c>
+      <c r="B31" s="67" t="inlineStr">
+        <is>
+          <t>Review and clean up global CSS (colors, fonts, spacing, typography)</t>
+        </is>
+      </c>
+      <c r="C31" s="68" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D31" s="68" t="n">
+        <v>46242</v>
+      </c>
       <c r="E31" s="30">
         <f>IF(OR(C31="",D31=""),"",NETWORKDAYS(C31,D31))</f>
         <v/>
       </c>
-      <c r="F31" s="66" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F31" s="69" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G31" s="31">
         <f>IF(F31="Completed",1,IF(F31="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H31" s="67">
+      <c r="H31" s="70">
         <f>IF(C31="","",C31+MOD(5-WEEKDAY(C31,2),7))</f>
         <v/>
       </c>
-      <c r="I31" s="53" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+      <c r="I31" s="67" t="inlineStr">
+        <is>
+          <t>Currently in progress — checking index.css theme tokens, base styles, and consistency with Tailwind usage across screens.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="53" t="inlineStr">
-        <is>
-          <t>6. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B32" s="53" t="inlineStr">
-        <is>
-          <t>Connect admin screens to live API (balances, conversion, reports)</t>
-        </is>
-      </c>
-      <c r="C32" s="65" t="n"/>
-      <c r="D32" s="65" t="n"/>
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>6. UI Polish &amp; Cleanup</t>
+        </is>
+      </c>
+      <c r="B32" s="67" t="inlineStr">
+        <is>
+          <t>Check and fix app shell layout (sidebar, top header, main content area)</t>
+        </is>
+      </c>
+      <c r="C32" s="68" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D32" s="68" t="n">
+        <v>46242</v>
+      </c>
       <c r="E32" s="30">
         <f>IF(OR(C32="",D32=""),"",NETWORKDAYS(C32,D32))</f>
         <v/>
       </c>
-      <c r="F32" s="66" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F32" s="69" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G32" s="31">
         <f>IF(F32="Completed",1,IF(F32="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H32" s="67">
+      <c r="H32" s="70">
         <f>IF(C32="","",C32+MOD(5-WEEKDAY(C32,2),7))</f>
         <v/>
       </c>
-      <c r="I32" s="53" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+      <c r="I32" s="67" t="inlineStr">
+        <is>
+          <t>Currently in progress — reviewing AppLayout, collapsible sidebar, header alignment, and page padding/overflow behavior.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="53" t="inlineStr">
-        <is>
-          <t>6. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B33" s="53" t="inlineStr">
-        <is>
-          <t>Joint frontend–backend smoke check once APIs are available</t>
-        </is>
-      </c>
-      <c r="C33" s="65" t="n"/>
-      <c r="D33" s="65" t="n"/>
+      <c r="A33" s="67" t="inlineStr">
+        <is>
+          <t>6. UI Polish &amp; Cleanup</t>
+        </is>
+      </c>
+      <c r="B33" s="67" t="inlineStr">
+        <is>
+          <t>Standardize screen layouts (tables, filter bars, forms, and reports)</t>
+        </is>
+      </c>
+      <c r="C33" s="68" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D33" s="68" t="n">
+        <v>46249</v>
+      </c>
       <c r="E33" s="30">
         <f>IF(OR(C33="",D33=""),"",NETWORKDAYS(C33,D33))</f>
         <v/>
       </c>
-      <c r="F33" s="66" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F33" s="69" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G33" s="31">
         <f>IF(F33="Completed",1,IF(F33="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H33" s="67">
+      <c r="H33" s="70">
         <f>IF(C33="","",C33+MOD(5-WEEKDAY(C33,2),7))</f>
         <v/>
       </c>
-      <c r="I33" s="53" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+      <c r="I33" s="67" t="inlineStr">
+        <is>
+          <t>Currently in progress — aligning filter control heights, table spacing, button placement, and responsive layout on list/form/report pages.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="54" t="inlineStr">
-        <is>
-          <t>7. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B34" s="54" t="inlineStr">
-        <is>
-          <t>Employee flow testing (file, edit, cancel, view history)</t>
-        </is>
-      </c>
-      <c r="C34" s="68" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D34" s="68" t="n"/>
+      <c r="A34" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B34" s="56" t="inlineStr">
+        <is>
+          <t>Connect frontend to backend API (base connection and shared data types)</t>
+        </is>
+      </c>
+      <c r="C34" s="71" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D34" s="71" t="n"/>
       <c r="E34" s="33">
         <f>IF(OR(C34="",D34=""),"",NETWORKDAYS(C34,D34))</f>
         <v/>
       </c>
-      <c r="F34" s="66" t="inlineStr">
+      <c r="F34" s="72" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2950,36 +3082,36 @@
         <f>IF(F34="Completed",1,IF(F34="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H34" s="69">
+      <c r="H34" s="73">
         <f>IF(C34="","",C34+MOD(5-WEEKDAY(C34,2),7))</f>
         <v/>
       </c>
-      <c r="I34" s="54" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+      <c r="I34" s="56" t="inlineStr">
+        <is>
+          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="54" t="inlineStr">
-        <is>
-          <t>7. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B35" s="54" t="inlineStr">
-        <is>
-          <t>Approver flow testing (approve, reject, team views)</t>
-        </is>
-      </c>
-      <c r="C35" s="68" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D35" s="68" t="n"/>
+      <c r="A35" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B35" s="56" t="inlineStr">
+        <is>
+          <t>Use portal cookies / session to identify the user (no separate login page)</t>
+        </is>
+      </c>
+      <c r="C35" s="71" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D35" s="71" t="n"/>
       <c r="E35" s="33">
         <f>IF(OR(C35="",D35=""),"",NETWORKDAYS(C35,D35))</f>
         <v/>
       </c>
-      <c r="F35" s="66" t="inlineStr">
+      <c r="F35" s="72" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -2988,36 +3120,34 @@
         <f>IF(F35="Completed",1,IF(F35="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H35" s="69">
+      <c r="H35" s="73">
         <f>IF(C35="","",C35+MOD(5-WEEKDAY(C35,2),7))</f>
         <v/>
       </c>
-      <c r="I35" s="54" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+      <c r="I35" s="56" t="inlineStr">
+        <is>
+          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known. Agreed with backend: cookies/session — no login screen.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="54" t="inlineStr">
-        <is>
-          <t>7. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B36" s="54" t="inlineStr">
-        <is>
-          <t>Admin flow testing (balances, conversion, reports)</t>
-        </is>
-      </c>
-      <c r="C36" s="68" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D36" s="68" t="n"/>
+      <c r="A36" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B36" s="56" t="inlineStr">
+        <is>
+          <t>Connect employee leave screens to live API (file, history, cancel, edit)</t>
+        </is>
+      </c>
+      <c r="C36" s="71" t="n"/>
+      <c r="D36" s="71" t="n"/>
       <c r="E36" s="33">
         <f>IF(OR(C36="",D36=""),"",NETWORKDAYS(C36,D36))</f>
         <v/>
       </c>
-      <c r="F36" s="66" t="inlineStr">
+      <c r="F36" s="72" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3026,36 +3156,34 @@
         <f>IF(F36="Completed",1,IF(F36="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H36" s="69">
+      <c r="H36" s="73">
         <f>IF(C36="","",C36+MOD(5-WEEKDAY(C36,2),7))</f>
         <v/>
       </c>
-      <c r="I36" s="54" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+      <c r="I36" s="56" t="inlineStr">
+        <is>
+          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="54" t="inlineStr">
-        <is>
-          <t>7. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B37" s="54" t="inlineStr">
-        <is>
-          <t>Mobile / responsive check on common screens</t>
-        </is>
-      </c>
-      <c r="C37" s="68" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D37" s="68" t="n"/>
+      <c r="A37" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B37" s="56" t="inlineStr">
+        <is>
+          <t>Connect approver / team screens to live API (inbox, approve, reject)</t>
+        </is>
+      </c>
+      <c r="C37" s="71" t="n"/>
+      <c r="D37" s="71" t="n"/>
       <c r="E37" s="33">
         <f>IF(OR(C37="",D37=""),"",NETWORKDAYS(C37,D37))</f>
         <v/>
       </c>
-      <c r="F37" s="66" t="inlineStr">
+      <c r="F37" s="72" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3064,36 +3192,34 @@
         <f>IF(F37="Completed",1,IF(F37="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H37" s="69">
+      <c r="H37" s="73">
         <f>IF(C37="","",C37+MOD(5-WEEKDAY(C37,2),7))</f>
         <v/>
       </c>
-      <c r="I37" s="54" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+      <c r="I37" s="56" t="inlineStr">
+        <is>
+          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="54" t="inlineStr">
-        <is>
-          <t>7. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B38" s="54" t="inlineStr">
-        <is>
-          <t>Fix issues found during testing</t>
-        </is>
-      </c>
-      <c r="C38" s="68" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D38" s="68" t="n"/>
+      <c r="A38" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B38" s="56" t="inlineStr">
+        <is>
+          <t>Connect admin screens to live API (balances, conversion, reports)</t>
+        </is>
+      </c>
+      <c r="C38" s="71" t="n"/>
+      <c r="D38" s="71" t="n"/>
       <c r="E38" s="33">
         <f>IF(OR(C38="",D38=""),"",NETWORKDAYS(C38,D38))</f>
         <v/>
       </c>
-      <c r="F38" s="66" t="inlineStr">
+      <c r="F38" s="72" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3102,74 +3228,72 @@
         <f>IF(F38="Completed",1,IF(F38="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H38" s="69">
+      <c r="H38" s="73">
         <f>IF(C38="","",C38+MOD(5-WEEKDAY(C38,2),7))</f>
         <v/>
       </c>
-      <c r="I38" s="54" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+      <c r="I38" s="56" t="inlineStr">
+        <is>
+          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="55" t="inlineStr">
-        <is>
-          <t>8. Documentation (after development)</t>
-        </is>
-      </c>
-      <c r="B39" s="55" t="inlineStr">
-        <is>
-          <t>Finalize frontend guide for the team (FRONTEND.md)</t>
-        </is>
-      </c>
-      <c r="C39" s="70" t="n">
+      <c r="A39" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B39" s="56" t="inlineStr">
+        <is>
+          <t>Joint frontend–backend smoke check once APIs are available</t>
+        </is>
+      </c>
+      <c r="C39" s="71" t="n"/>
+      <c r="D39" s="71" t="n"/>
+      <c r="E39" s="33">
+        <f>IF(OR(C39="",D39=""),"",NETWORKDAYS(C39,D39))</f>
+        <v/>
+      </c>
+      <c r="F39" s="72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G39" s="34">
+        <f>IF(F39="Completed",1,IF(F39="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H39" s="73">
+        <f>IF(C39="","",C39+MOD(5-WEEKDAY(C39,2),7))</f>
+        <v/>
+      </c>
+      <c r="I39" s="56" t="inlineStr">
+        <is>
+          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B40" s="57" t="inlineStr">
+        <is>
+          <t>Employee flow testing (file, edit, cancel, view history)</t>
+        </is>
+      </c>
+      <c r="C40" s="74" t="n">
         <v>46266</v>
       </c>
-      <c r="D39" s="70" t="n"/>
-      <c r="E39" s="36">
-        <f>IF(OR(C39="",D39=""),"",NETWORKDAYS(C39,D39))</f>
-        <v/>
-      </c>
-      <c r="F39" s="66" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G39" s="37">
-        <f>IF(F39="Completed",1,IF(F39="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H39" s="71">
-        <f>IF(C39="","",C39+MOD(5-WEEKDAY(C39,2),7))</f>
-        <v/>
-      </c>
-      <c r="I39" s="55" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="55" t="inlineStr">
-        <is>
-          <t>8. Documentation (after development)</t>
-        </is>
-      </c>
-      <c r="B40" s="55" t="inlineStr">
-        <is>
-          <t>Prepare short demo / walkthrough notes for stakeholders</t>
-        </is>
-      </c>
-      <c r="C40" s="70" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D40" s="70" t="n"/>
+      <c r="D40" s="74" t="n"/>
       <c r="E40" s="36">
         <f>IF(OR(C40="",D40=""),"",NETWORKDAYS(C40,D40))</f>
         <v/>
       </c>
-      <c r="F40" s="66" t="inlineStr">
+      <c r="F40" s="72" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3178,36 +3302,36 @@
         <f>IF(F40="Completed",1,IF(F40="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H40" s="71">
+      <c r="H40" s="75">
         <f>IF(C40="","",C40+MOD(5-WEEKDAY(C40,2),7))</f>
         <v/>
       </c>
-      <c r="I40" s="55" t="inlineStr">
+      <c r="I40" s="57" t="inlineStr">
         <is>
           <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="55" t="inlineStr">
-        <is>
-          <t>8. Documentation (after development)</t>
-        </is>
-      </c>
-      <c r="B41" s="55" t="inlineStr">
-        <is>
-          <t>Handover checklist (how to run, deploy, and who owns what)</t>
-        </is>
-      </c>
-      <c r="C41" s="70" t="n">
+      <c r="A41" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B41" s="57" t="inlineStr">
+        <is>
+          <t>Approver flow testing (approve, reject, team views)</t>
+        </is>
+      </c>
+      <c r="C41" s="74" t="n">
         <v>46266</v>
       </c>
-      <c r="D41" s="70" t="n"/>
+      <c r="D41" s="74" t="n"/>
       <c r="E41" s="36">
         <f>IF(OR(C41="",D41=""),"",NETWORKDAYS(C41,D41))</f>
         <v/>
       </c>
-      <c r="F41" s="66" t="inlineStr">
+      <c r="F41" s="72" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3216,29 +3340,257 @@
         <f>IF(F41="Completed",1,IF(F41="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H41" s="71">
+      <c r="H41" s="75">
         <f>IF(C41="","",C41+MOD(5-WEEKDAY(C41,2),7))</f>
         <v/>
       </c>
-      <c r="I41" s="55" t="inlineStr">
+      <c r="I41" s="57" t="inlineStr">
         <is>
           <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B42" s="57" t="inlineStr">
+        <is>
+          <t>Admin flow testing (balances, conversion, reports)</t>
+        </is>
+      </c>
+      <c r="C42" s="74" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D42" s="74" t="n"/>
+      <c r="E42" s="36">
+        <f>IF(OR(C42="",D42=""),"",NETWORKDAYS(C42,D42))</f>
+        <v/>
+      </c>
+      <c r="F42" s="72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G42" s="37">
+        <f>IF(F42="Completed",1,IF(F42="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H42" s="75">
+        <f>IF(C42="","",C42+MOD(5-WEEKDAY(C42,2),7))</f>
+        <v/>
+      </c>
+      <c r="I42" s="57" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B43" s="57" t="inlineStr">
+        <is>
+          <t>Mobile / responsive check on common screens</t>
+        </is>
+      </c>
+      <c r="C43" s="74" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D43" s="74" t="n"/>
+      <c r="E43" s="36">
+        <f>IF(OR(C43="",D43=""),"",NETWORKDAYS(C43,D43))</f>
+        <v/>
+      </c>
+      <c r="F43" s="72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G43" s="37">
+        <f>IF(F43="Completed",1,IF(F43="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H43" s="75">
+        <f>IF(C43="","",C43+MOD(5-WEEKDAY(C43,2),7))</f>
+        <v/>
+      </c>
+      <c r="I43" s="57" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B44" s="57" t="inlineStr">
+        <is>
+          <t>Fix issues found during testing</t>
+        </is>
+      </c>
+      <c r="C44" s="74" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D44" s="74" t="n"/>
+      <c r="E44" s="36">
+        <f>IF(OR(C44="",D44=""),"",NETWORKDAYS(C44,D44))</f>
+        <v/>
+      </c>
+      <c r="F44" s="72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G44" s="37">
+        <f>IF(F44="Completed",1,IF(F44="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H44" s="75">
+        <f>IF(C44="","",C44+MOD(5-WEEKDAY(C44,2),7))</f>
+        <v/>
+      </c>
+      <c r="I44" s="57" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="58" t="inlineStr">
+        <is>
+          <t>9. Documentation (after development)</t>
+        </is>
+      </c>
+      <c r="B45" s="58" t="inlineStr">
+        <is>
+          <t>Finalize frontend guide for the team (FRONTEND.md)</t>
+        </is>
+      </c>
+      <c r="C45" s="76" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D45" s="76" t="n"/>
+      <c r="E45" s="39">
+        <f>IF(OR(C45="",D45=""),"",NETWORKDAYS(C45,D45))</f>
+        <v/>
+      </c>
+      <c r="F45" s="72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G45" s="40">
+        <f>IF(F45="Completed",1,IF(F45="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H45" s="77">
+        <f>IF(C45="","",C45+MOD(5-WEEKDAY(C45,2),7))</f>
+        <v/>
+      </c>
+      <c r="I45" s="58" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="58" t="inlineStr">
+        <is>
+          <t>9. Documentation (after development)</t>
+        </is>
+      </c>
+      <c r="B46" s="58" t="inlineStr">
+        <is>
+          <t>Prepare short demo / walkthrough notes for stakeholders</t>
+        </is>
+      </c>
+      <c r="C46" s="76" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D46" s="76" t="n"/>
+      <c r="E46" s="39">
+        <f>IF(OR(C46="",D46=""),"",NETWORKDAYS(C46,D46))</f>
+        <v/>
+      </c>
+      <c r="F46" s="72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G46" s="40">
+        <f>IF(F46="Completed",1,IF(F46="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H46" s="77">
+        <f>IF(C46="","",C46+MOD(5-WEEKDAY(C46,2),7))</f>
+        <v/>
+      </c>
+      <c r="I46" s="58" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="58" t="inlineStr">
+        <is>
+          <t>9. Documentation (after development)</t>
+        </is>
+      </c>
+      <c r="B47" s="58" t="inlineStr">
+        <is>
+          <t>Handover checklist (how to run, deploy, and who owns what)</t>
+        </is>
+      </c>
+      <c r="C47" s="76" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D47" s="76" t="n"/>
+      <c r="E47" s="39">
+        <f>IF(OR(C47="",D47=""),"",NETWORKDAYS(C47,D47))</f>
+        <v/>
+      </c>
+      <c r="F47" s="72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G47" s="40">
+        <f>IF(F47="Completed",1,IF(F47="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H47" s="77">
+        <f>IF(C47="","",C47+MOD(5-WEEKDAY(C47,2),7))</f>
+        <v/>
+      </c>
+      <c r="I47" s="58" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Commitment: frontend DEVELOPMENT finished by end of August (weekdays = NETWORKDAYS). Backend Integration has TBD end dates (teams work separately — fill dates when known). Testing and Documentation start after development (from Sep 2026); end dates TBD. No login page — portal cookies/session with backend.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I41"/>
+  <autoFilter ref="A1:I47"/>
   <mergeCells count="1">
-    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A49:I49"/>
   </mergeCells>
-  <conditionalFormatting sqref="G2:G41">
+  <conditionalFormatting sqref="G2:G47">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -3251,7 +3603,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Completed,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3279,168 +3631,168 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="72" t="inlineStr"/>
+      <c r="A2" s="78" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="73" t="inlineStr">
+      <c r="A3" s="79" t="inlineStr">
         <is>
           <t>August commitment</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="78" t="inlineStr">
         <is>
           <t>Only frontend DEVELOPMENT is committed to finish by end of August.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="72" t="inlineStr">
+      <c r="A5" s="78" t="inlineStr">
         <is>
           <t>Testing and documentation come AFTER development (start ~1 Sep; end dates TBD).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="72" t="inlineStr">
+      <c r="A6" s="78" t="inlineStr">
         <is>
           <t>Backend Integration is listed with TBD dates — teams work separately for now.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="72" t="inlineStr"/>
+      <c r="A7" s="78" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="73" t="inlineStr">
+      <c r="A8" s="79" t="inlineStr">
         <is>
           <t>For leaders / managers</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="72" t="inlineStr">
-        <is>
-          <t>1. Dashboard — overall % and section progress (also see Development progress for sections 1–5).</t>
+      <c r="A9" s="78" t="inlineStr">
+        <is>
+          <t>1. Dashboard — overall % and section progress (also see Development progress for sections 1–6).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="72" t="inlineStr">
+      <c r="A10" s="78" t="inlineStr">
         <is>
           <t>2. Tentative Schedule — development phases through August; backend/testing/docs called out as TBD/after.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="72" t="inlineStr">
+      <c r="A11" s="78" t="inlineStr">
         <is>
           <t>3. Progress Tracker — update Status here.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="72" t="inlineStr"/>
+      <c r="A12" s="78" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="73" t="inlineStr">
+      <c r="A13" s="79" t="inlineStr">
         <is>
           <t>For the development team</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="72" t="inlineStr">
+      <c r="A14" s="78" t="inlineStr">
         <is>
           <t>1. Change Status on Progress Tracker (dropdown).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="72" t="inlineStr">
+      <c r="A15" s="78" t="inlineStr">
         <is>
           <t>2. For Backend Integration / Testing / Documentation: fill Start and End dates when known.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="72" t="inlineStr">
+      <c r="A16" s="78" t="inlineStr">
         <is>
           <t>3. Keyword for Cursor: Update the leader tracker from the code</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="72" t="inlineStr"/>
+      <c r="A17" s="78" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="73" t="inlineStr">
+      <c r="A18" s="79" t="inlineStr">
         <is>
           <t>Workdays</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="72" t="inlineStr">
+      <c r="A19" s="78" t="inlineStr">
         <is>
           <t>Days (weekdays) uses NETWORKDAYS when both Start and End are filled (Mon–Fri only).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="72" t="inlineStr"/>
+      <c r="A20" s="78" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="73" t="inlineStr">
+      <c r="A21" s="79" t="inlineStr">
         <is>
           <t>Authentication</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="72" t="inlineStr">
+      <c r="A22" s="78" t="inlineStr">
         <is>
           <t>No login page. User identity via portal cookies/session with the backend partner.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="72" t="inlineStr"/>
+      <c r="A23" s="78" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="73" t="inlineStr">
+      <c r="A24" s="79" t="inlineStr">
         <is>
           <t>Status meanings</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="72" t="inlineStr">
+      <c r="A25" s="78" t="inlineStr">
         <is>
           <t>Completed / In Progress / Not Started / Blocked</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="72" t="inlineStr">
+      <c r="A26" s="78" t="inlineStr">
         <is>
           <t>Scoring: Completed = 100%, In Progress = 50%, else 0%.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="72" t="inlineStr"/>
+      <c r="A27" s="78" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="73" t="inlineStr">
+      <c r="A28" s="79" t="inlineStr">
         <is>
           <t>Related files</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="72" t="inlineStr">
+      <c r="A29" s="78" t="inlineStr">
         <is>
           <t>docs/FRONTEND.md</t>
         </is>

</xml_diff>

<commit_message>
Update project timelines and enhance task descriptions in the tracker. Adjust button styles for better hover effects
</commit_message>
<xml_diff>
--- a/docs/FRONTEND_LEADER_TRACKER.xlsx
+++ b/docs/FRONTEND_LEADER_TRACKER.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tentative Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progress Tracker" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tentative Schedule" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Progress Tracker'!$A$1:$I$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Progress Tracker'!$A$1:$I$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -141,17 +141,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2D5F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAD1DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -218,7 +218,7 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -230,7 +230,7 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -267,18 +267,18 @@
     <xf numFmtId="9" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -313,8 +313,8 @@
     <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -339,22 +339,22 @@
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -761,14 +761,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Backend Integration is listed separately — schedule depends on the backend partner. No separate login page (portal cookies/session). Days = weekdays only when both dates are set.</t>
+          <t>Backend Integration is underway (employee + key approver screens on live API). Production auth is portal cookies/session (dev-only employee ID entry for local testing). Days = weekdays only when both dates are set.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Last aligned to codebase: 2026-07-30 — all screens built with mock data; currently polishing CSS and layouts (section 6); cookie/session and live API not wired yet.</t>
+          <t>Last aligned to codebase: 2026-08-13 — live API wired for auth + employee + key approver flows; admin still mock; CODEBASE REVIEW AND CLEANUP STILL IN PROGRESS (section 6).</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
         <v>46233</v>
       </c>
       <c r="C9" s="53" t="n">
-        <v>46249</v>
+        <v>46256</v>
       </c>
       <c r="D9" s="18">
         <f>NETWORKDAYS(B9,C9)</f>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="E9" s="52" t="inlineStr">
         <is>
-          <t>CSS review, layout checks, and consistent spacing across screens.</t>
+          <t>CSS/layout review STILL IN PROGRESS; shared leave components and empty states landed.</t>
         </is>
       </c>
       <c r="F9" s="53">
@@ -1411,12 +1411,12 @@
     <row r="15">
       <c r="A15" s="56" t="inlineStr">
         <is>
-          <t>Backend integration (parallel / TBD)</t>
+          <t>Backend integration (in progress)</t>
         </is>
       </c>
       <c r="B15" s="56" t="inlineStr">
         <is>
-          <t>Ongoing with backend partner — no fixed day count yet. Update when APIs and cookie/session are ready.</t>
+          <t>Employee + key approver APIs wired (as of 2026-08-13). Admin APIs and remaining team screens still TBD.</t>
         </is>
       </c>
     </row>
@@ -1495,11 +1495,11 @@
     <row r="23">
       <c r="A23" s="59" t="inlineStr">
         <is>
-          <t>Reusable UI + employee screens underway</t>
+          <t>Admin screens usable (UI) — done early</t>
         </is>
       </c>
       <c r="B23" s="60" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="C23" s="60">
         <f>B23+MOD(5-WEEKDAY(B23,2),7)</f>
@@ -1507,18 +1507,18 @@
       </c>
       <c r="D23" s="59" t="inlineStr">
         <is>
-          <t>2–3</t>
+          <t>5. Admin Features</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="59" t="inlineStr">
         <is>
-          <t>Employee filing &amp; history usable (UI)</t>
+          <t>UI polish &amp; layout cleanup underway</t>
         </is>
       </c>
       <c r="B24" s="60" t="n">
-        <v>46247</v>
+        <v>46233</v>
       </c>
       <c r="C24" s="60">
         <f>B24+MOD(5-WEEKDAY(B24,2),7)</f>
@@ -1526,18 +1526,18 @@
       </c>
       <c r="D24" s="59" t="inlineStr">
         <is>
-          <t>3. Employee Features</t>
+          <t>6. UI Polish &amp; Cleanup</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="59" t="inlineStr">
         <is>
-          <t>Approver approve/reject usable (UI)</t>
+          <t>Notifications + error pages</t>
         </is>
       </c>
       <c r="B25" s="60" t="n">
-        <v>46252</v>
+        <v>46234</v>
       </c>
       <c r="C25" s="60">
         <f>B25+MOD(5-WEEKDAY(B25,2),7)</f>
@@ -1545,18 +1545,18 @@
       </c>
       <c r="D25" s="59" t="inlineStr">
         <is>
-          <t>4. Approver / Team</t>
+          <t>2. Core App Shell</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="59" t="inlineStr">
         <is>
-          <t>Admin screens usable (UI) — done early</t>
+          <t>Employee + approver live API wiring started</t>
         </is>
       </c>
       <c r="B26" s="60" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="C26" s="60">
         <f>B26+MOD(5-WEEKDAY(B26,2),7)</f>
@@ -1564,18 +1564,18 @@
       </c>
       <c r="D26" s="59" t="inlineStr">
         <is>
-          <t>5. Admin Features</t>
+          <t>7. Backend Integration</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="59" t="inlineStr">
         <is>
-          <t>Admin screens target (original plan)</t>
+          <t>Codebase review &amp; cleanup still in progress</t>
         </is>
       </c>
       <c r="B27" s="60" t="n">
-        <v>46262</v>
+        <v>46247</v>
       </c>
       <c r="C27" s="60">
         <f>B27+MOD(5-WEEKDAY(B27,2),7)</f>
@@ -1583,18 +1583,18 @@
       </c>
       <c r="D27" s="59" t="inlineStr">
         <is>
-          <t>5. Admin Features</t>
+          <t>6. UI Polish &amp; Cleanup</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="59" t="inlineStr">
         <is>
-          <t>UI polish &amp; layout cleanup underway</t>
+          <t>Live auth + employee/approver APIs in progress</t>
         </is>
       </c>
       <c r="B28" s="60" t="n">
-        <v>46233</v>
+        <v>46247</v>
       </c>
       <c r="C28" s="60">
         <f>B28+MOD(5-WEEKDAY(B28,2),7)</f>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D28" s="59" t="inlineStr">
         <is>
-          <t>6. UI Polish &amp; Cleanup</t>
+          <t>7. Backend Integration</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D29" s="59" t="inlineStr">
         <is>
-          <t>Sections 1–6</t>
+          <t>Sections 1–7</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="B36" s="59" t="inlineStr">
         <is>
-          <t>CSS and layout cleanup in progress across screens</t>
+          <t>CSS/layout cleanup in progress; shared leave detail layout improvements</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B37" s="59" t="inlineStr">
         <is>
-          <t>Layout polish wrapping up; ready for backend hookup when APIs are available</t>
+          <t>Codebase review still in progress; live auth + employee/approver APIs wired</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B38" s="59" t="inlineStr">
         <is>
-          <t>Approver UI in place; admin screens underway</t>
+          <t>Continue UI polish + finish remaining API wiring (team calendar, admin)</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B39" s="59" t="inlineStr">
         <is>
-          <t>Admin UI in progress / wrapping up</t>
+          <t>Wrap remaining polish and admin API work before Aug commitment</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1896,7 +1896,11 @@
         <f>IF(C4="","",C4+MOD(5-WEEKDAY(C4,2),7))</f>
         <v/>
       </c>
-      <c r="I4" s="44" t="inlineStr"/>
+      <c r="I4" s="44" t="inlineStr">
+        <is>
+          <t>Routes include RequireAuth / RequireCapability gates and error preview paths.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="52" t="inlineStr">
@@ -1949,7 +1953,7 @@
         <v>46224</v>
       </c>
       <c r="D6" s="53" t="n">
-        <v>46225</v>
+        <v>46247</v>
       </c>
       <c r="E6" s="18">
         <f>IF(OR(C6="",D6=""),"",NETWORKDAYS(C6,D6))</f>
@@ -1970,7 +1974,7 @@
       </c>
       <c r="I6" s="52" t="inlineStr">
         <is>
-          <t>Role-based sidebar works. Dev-only role preview remains until portal cookies/session are wired.</t>
+          <t>Sidebar + RequireCapability use live roles from /api/me (approver/admin). Dev persona switcher removed as auth is wired.</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1993,7 @@
         <v>46225</v>
       </c>
       <c r="D7" s="53" t="n">
-        <v>46233</v>
+        <v>46247</v>
       </c>
       <c r="E7" s="18">
         <f>IF(OR(C7="",D7=""),"",NETWORKDAYS(C7,D7))</f>
@@ -2010,7 +2014,7 @@
       </c>
       <c r="I7" s="52" t="inlineStr">
         <is>
-          <t>Built: StatusBadge, FilterSelect, Pagination, Button, Modal, ConfirmReasonModal, AttachmentPreviewModal, SuccessDialog, Skeleton, form fields, MonthYearPickerField, YearPickerField, EmployeeMultiSelect, tableStyles, admin-specific components.</t>
+          <t>Built: StatusBadge, FilterSelect, Pagination, Button, Modal, ConfirmReasonModal, AttachmentPreviewModal, SuccessDialog, Skeleton, EmptyState, TableEmptyRow, SortableHeader, ListTabButton, PageBackLink, NotificationPanel, form fields, shared leave panels, tableStyles/tableLayout, admin components.</t>
         </is>
       </c>
     </row>
@@ -2050,7 +2054,7 @@
       </c>
       <c r="I8" s="52" t="inlineStr">
         <is>
-          <t>Sidebar collapses to icon-only mode with flyout submenus, tooltips, and localStorage preference. Top header toggle wired in AppLayout.</t>
+          <t>Collapsible sidebar with flyouts, localStorage preference, and responsive/mobile behavior (useMediaQuery).</t>
         </is>
       </c>
     </row>
@@ -2062,14 +2066,14 @@
       </c>
       <c r="B9" s="52" t="inlineStr">
         <is>
-          <t>Replace temporary placeholder pages with real screens</t>
+          <t>In-app notifications panel (header bell)</t>
         </is>
       </c>
       <c r="C9" s="53" t="n">
-        <v>46225</v>
+        <v>46234</v>
       </c>
       <c r="D9" s="53" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E9" s="18">
         <f>IF(OR(C9="",D9=""),"",NETWORKDAYS(C9,D9))</f>
@@ -2090,87 +2094,87 @@
       </c>
       <c r="I9" s="52" t="inlineStr">
         <is>
-          <t>All employee, approver/team, and admin routes now have real page components. PagePlaceholder is no longer used in routing.</t>
+          <t>NotificationPanel in TopHeader (unread filter, mark read). Still uses mock notifications until a notifications API is available.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="46" t="inlineStr">
-        <is>
-          <t>3. Employee Features</t>
-        </is>
-      </c>
-      <c r="B10" s="46" t="inlineStr">
-        <is>
-          <t>Employee dashboard: leave balances and recent requests</t>
-        </is>
-      </c>
-      <c r="C10" s="47" t="n">
+      <c r="A10" s="52" t="inlineStr">
+        <is>
+          <t>2. Core App Shell</t>
+        </is>
+      </c>
+      <c r="B10" s="52" t="inlineStr">
+        <is>
+          <t>Error and system feedback pages (401, 403, 404, 409, 500, 503, offline)</t>
+        </is>
+      </c>
+      <c r="C10" s="53" t="n">
+        <v>46234</v>
+      </c>
+      <c r="D10" s="53" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E10" s="18">
+        <f>IF(OR(C10="",D10=""),"",NETWORKDAYS(C10,D10))</f>
+        <v/>
+      </c>
+      <c r="F10" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G10" s="19">
+        <f>IF(F10="Completed",1,IF(F10="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H10" s="63">
+        <f>IF(C10="","",C10+MOD(5-WEEKDAY(C10,2),7))</f>
+        <v/>
+      </c>
+      <c r="I10" s="52" t="inlineStr">
+        <is>
+          <t>Shared ErrorPage layout + dedicated routes. Catch-all invalid URLs show NotFound without redirecting away from the URL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="52" t="inlineStr">
+        <is>
+          <t>2. Core App Shell</t>
+        </is>
+      </c>
+      <c r="B11" s="52" t="inlineStr">
+        <is>
+          <t>Replace temporary placeholder pages with real screens</t>
+        </is>
+      </c>
+      <c r="C11" s="53" t="n">
         <v>46225</v>
       </c>
-      <c r="D10" s="47" t="n">
-        <v>46225</v>
-      </c>
-      <c r="E10" s="21">
-        <f>IF(OR(C10="",D10=""),"",NETWORKDAYS(C10,D10))</f>
-        <v/>
-      </c>
-      <c r="F10" s="36" t="inlineStr">
+      <c r="D11" s="53" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E11" s="18">
+        <f>IF(OR(C11="",D11=""),"",NETWORKDAYS(C11,D11))</f>
+        <v/>
+      </c>
+      <c r="F11" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="G10" s="22">
-        <f>IF(F10="Completed",1,IF(F10="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H10" s="64">
-        <f>IF(C10="","",C10+MOD(5-WEEKDAY(C10,2),7))</f>
-        <v/>
-      </c>
-      <c r="I10" s="46" t="inlineStr">
-        <is>
-          <t>UI complete (balances, reserved credits, filters, pagination). Uses mock data until Backend Integration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="46" t="inlineStr">
-        <is>
-          <t>3. Employee Features</t>
-        </is>
-      </c>
-      <c r="B11" s="46" t="inlineStr">
-        <is>
-          <t>File leave request (dates, leave type, reason, attachment)</t>
-        </is>
-      </c>
-      <c r="C11" s="47" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D11" s="47" t="n">
-        <v>46226</v>
-      </c>
-      <c r="E11" s="21">
-        <f>IF(OR(C11="",D11=""),"",NETWORKDAYS(C11,D11))</f>
-        <v/>
-      </c>
-      <c r="F11" s="36" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="G11" s="22">
+      <c r="G11" s="19">
         <f>IF(F11="Completed",1,IF(F11="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H11" s="64">
+      <c r="H11" s="63">
         <f>IF(C11="","",C11+MOD(5-WEEKDAY(C11,2),7))</f>
         <v/>
       </c>
-      <c r="I11" s="46" t="inlineStr">
-        <is>
-          <t>Apply Leave page is built with employee info, leave type/day type, date range, reason, attachment rules, duration preview, confirm modal, and success dialog. Uses mock submit until Backend Integration.</t>
+      <c r="I11" s="52" t="inlineStr">
+        <is>
+          <t>All feature routes use real pages. PagePlaceholder and unused icons removed. Empty lists use EmptyState / TableEmptyRow.</t>
         </is>
       </c>
     </row>
@@ -2182,14 +2186,14 @@
       </c>
       <c r="B12" s="46" t="inlineStr">
         <is>
-          <t>Show unpaid leave (LWOP) warning when credits are not enough</t>
+          <t>Employee dashboard: leave balances and recent requests</t>
         </is>
       </c>
       <c r="C12" s="47" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="D12" s="47" t="n">
-        <v>46226</v>
+        <v>46247</v>
       </c>
       <c r="E12" s="21">
         <f>IF(OR(C12="",D12=""),"",NETWORKDAYS(C12,D12))</f>
@@ -2210,7 +2214,7 @@
       </c>
       <c r="I12" s="46" t="inlineStr">
         <is>
-          <t>LWOP / remaining-balance warning is shown in filing forms using mock remaining-day logic.</t>
+          <t>UI complete; now loads live balances and leave list via useMyBalances / useMyLeaves (SWR).</t>
         </is>
       </c>
     </row>
@@ -2222,14 +2226,14 @@
       </c>
       <c r="B13" s="46" t="inlineStr">
         <is>
-          <t>Leave request details: status, approvals needed, and activity history</t>
+          <t>File leave request (dates, leave type, reason, attachment)</t>
         </is>
       </c>
       <c r="C13" s="47" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="D13" s="47" t="n">
-        <v>46225</v>
+        <v>46247</v>
       </c>
       <c r="E13" s="21">
         <f>IF(OR(C13="",D13=""),"",NETWORKDAYS(C13,D13))</f>
@@ -2250,7 +2254,7 @@
       </c>
       <c r="I13" s="46" t="inlineStr">
         <is>
-          <t>UI complete: leave info, approval progress/requirements, approver list, attachments, conversion view. Mock data; activity timeline not a separate log yet.</t>
+          <t>Apply Leave submits via createLeave API; holiday dates from live holidays hook. Multi-file attachments supported.</t>
         </is>
       </c>
     </row>
@@ -2262,14 +2266,14 @@
       </c>
       <c r="B14" s="46" t="inlineStr">
         <is>
-          <t>Activity log / leave history with filters</t>
+          <t>Show unpaid leave (LWOP) warning when credits are not enough</t>
         </is>
       </c>
       <c r="C14" s="47" t="n">
         <v>46226</v>
       </c>
       <c r="D14" s="47" t="n">
-        <v>46226</v>
+        <v>46247</v>
       </c>
       <c r="E14" s="21">
         <f>IF(OR(C14="",D14=""),"",NETWORKDAYS(C14,D14))</f>
@@ -2290,7 +2294,7 @@
       </c>
       <c r="I14" s="46" t="inlineStr">
         <is>
-          <t>Activity Log page exists with filtering, sorting, pagination, and mock activity data.</t>
+          <t>LWOP / remaining-balance warning shown in filing forms using live balance data where available.</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2306,7 @@
       </c>
       <c r="B15" s="46" t="inlineStr">
         <is>
-          <t>Edit leave request (only while still waiting for first approval)</t>
+          <t>Leave request details: status, approvals needed, and activity history</t>
         </is>
       </c>
       <c r="C15" s="47" t="n">
@@ -2330,7 +2334,7 @@
       </c>
       <c r="I15" s="46" t="inlineStr">
         <is>
-          <t>Edit Leave page exists with date/day-type/reason editing, weekday duration recalculation, lead-time validation, confirm modal, and rules from details page. Uses mock save until Backend Integration.</t>
+          <t>Details page uses live useLeaveDetail + Approval Details table. Cancel calls live cancelLeave API.</t>
         </is>
       </c>
     </row>
@@ -2342,11 +2346,11 @@
       </c>
       <c r="B16" s="46" t="inlineStr">
         <is>
-          <t>Cancel leave request (with required reason)</t>
+          <t>Activity log / leave history with filters</t>
         </is>
       </c>
       <c r="C16" s="47" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="D16" s="47" t="n">
         <v>46247</v>
@@ -2370,7 +2374,7 @@
       </c>
       <c r="I16" s="46" t="inlineStr">
         <is>
-          <t>Cancel flow is present on details page with required-reason modal and success state. Uses mock action until Backend Integration.</t>
+          <t>Activity Log page wired to live useActivities API with filters, sorting, and pagination.</t>
         </is>
       </c>
     </row>
@@ -2382,14 +2386,14 @@
       </c>
       <c r="B17" s="46" t="inlineStr">
         <is>
-          <t>Request vacation-to-sick leave conversion (upload medical certificate)</t>
+          <t>Edit leave request (only while still waiting for first approval)</t>
         </is>
       </c>
       <c r="C17" s="47" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="D17" s="47" t="n">
-        <v>46226</v>
+        <v>46247</v>
       </c>
       <c r="E17" s="21">
         <f>IF(OR(C17="",D17=""),"",NETWORKDAYS(C17,D17))</f>
@@ -2410,87 +2414,87 @@
       </c>
       <c r="I17" s="46" t="inlineStr">
         <is>
-          <t>Conversion page exists with reason + medical certificate upload, eligibility rules, confirm modal, and mock submission.</t>
+          <t>Edit Leave loads live detail and saves via updateLeave API; holiday dates from live hook.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="48" t="inlineStr">
-        <is>
-          <t>4. Approver / Team Features</t>
-        </is>
-      </c>
-      <c r="B18" s="48" t="inlineStr">
-        <is>
-          <t>Approver inbox: list of leave requests waiting for action</t>
-        </is>
-      </c>
-      <c r="C18" s="49" t="n">
+      <c r="A18" s="46" t="inlineStr">
+        <is>
+          <t>3. Employee Features</t>
+        </is>
+      </c>
+      <c r="B18" s="46" t="inlineStr">
+        <is>
+          <t>Cancel leave request (with required reason)</t>
+        </is>
+      </c>
+      <c r="C18" s="47" t="n">
+        <v>46225</v>
+      </c>
+      <c r="D18" s="47" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E18" s="21">
+        <f>IF(OR(C18="",D18=""),"",NETWORKDAYS(C18,D18))</f>
+        <v/>
+      </c>
+      <c r="F18" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G18" s="22">
+        <f>IF(F18="Completed",1,IF(F18="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H18" s="64">
+        <f>IF(C18="","",C18+MOD(5-WEEKDAY(C18,2),7))</f>
+        <v/>
+      </c>
+      <c r="I18" s="46" t="inlineStr">
+        <is>
+          <t>Cancel flow on details page with required reason; live cancelLeave + cache revalidation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="46" t="inlineStr">
+        <is>
+          <t>3. Employee Features</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>Request vacation-to-sick leave conversion (upload medical certificate)</t>
+        </is>
+      </c>
+      <c r="C19" s="47" t="n">
         <v>46226</v>
       </c>
-      <c r="D18" s="49" t="n">
-        <v>46226</v>
-      </c>
-      <c r="E18" s="24">
-        <f>IF(OR(C18="",D18=""),"",NETWORKDAYS(C18,D18))</f>
-        <v/>
-      </c>
-      <c r="F18" s="36" t="inlineStr">
+      <c r="D19" s="47" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E19" s="21">
+        <f>IF(OR(C19="",D19=""),"",NETWORKDAYS(C19,D19))</f>
+        <v/>
+      </c>
+      <c r="F19" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="G18" s="25">
-        <f>IF(F18="Completed",1,IF(F18="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H18" s="65">
-        <f>IF(C18="","",C18+MOD(5-WEEKDAY(C18,2),7))</f>
-        <v/>
-      </c>
-      <c r="I18" s="48" t="inlineStr">
-        <is>
-          <t>Leave Approvals page exists with pending/all tabs, search, filters, sorting, pagination, and mock queue data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="48" t="inlineStr">
-        <is>
-          <t>4. Approver / Team Features</t>
-        </is>
-      </c>
-      <c r="B19" s="48" t="inlineStr">
-        <is>
-          <t>Approve or reject leave (reject requires remarks)</t>
-        </is>
-      </c>
-      <c r="C19" s="49" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D19" s="49" t="n">
-        <v>46226</v>
-      </c>
-      <c r="E19" s="24">
-        <f>IF(OR(C19="",D19=""),"",NETWORKDAYS(C19,D19))</f>
-        <v/>
-      </c>
-      <c r="F19" s="36" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="G19" s="25">
+      <c r="G19" s="22">
         <f>IF(F19="Completed",1,IF(F19="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H19" s="65">
+      <c r="H19" s="64">
         <f>IF(C19="","",C19+MOD(5-WEEKDAY(C19,2),7))</f>
         <v/>
       </c>
-      <c r="I19" s="48" t="inlineStr">
-        <is>
-          <t>Review page supports approve/reject actions, required rejection reason, confirmation modals, and success dialogs. Uses mock actions until Backend Integration.</t>
+      <c r="I19" s="46" t="inlineStr">
+        <is>
+          <t>Conversion page uses live leave detail and requestConversion API (multipart med cert).</t>
         </is>
       </c>
     </row>
@@ -2502,14 +2506,14 @@
       </c>
       <c r="B20" s="48" t="inlineStr">
         <is>
-          <t>Show clear approval progress (who still needs to act)</t>
+          <t>Approver inbox: list of leave requests waiting for action</t>
         </is>
       </c>
       <c r="C20" s="49" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="D20" s="49" t="n">
-        <v>46252</v>
+        <v>46247</v>
       </c>
       <c r="E20" s="24">
         <f>IF(OR(C20="",D20=""),"",NETWORKDAYS(C20,D20))</f>
@@ -2530,7 +2534,7 @@
       </c>
       <c r="I20" s="48" t="inlineStr">
         <is>
-          <t>Approval progress bars, requirement checklist, and approver status tables are built on employee details and approver review pages.</t>
+          <t>Leave Approvals inbox uses live usePendingApprovals / useApprovals (pending + all tabs).</t>
         </is>
       </c>
     </row>
@@ -2542,14 +2546,14 @@
       </c>
       <c r="B21" s="48" t="inlineStr">
         <is>
-          <t>File leave on behalf of a team member</t>
+          <t>Approve or reject leave (reject requires remarks)</t>
         </is>
       </c>
       <c r="C21" s="49" t="n">
         <v>46226</v>
       </c>
       <c r="D21" s="49" t="n">
-        <v>46226</v>
+        <v>46247</v>
       </c>
       <c r="E21" s="24">
         <f>IF(OR(C21="",D21=""),"",NETWORKDAYS(C21,D21))</f>
@@ -2570,7 +2574,7 @@
       </c>
       <c r="I21" s="48" t="inlineStr">
         <is>
-          <t>File Leave for Member page exists with member selection, leave form, LWOP warning, attachment rules, confirm modal, and mock submit.</t>
+          <t>Review page calls live approveLeave / rejectLeave APIs with confirmation modals.</t>
         </is>
       </c>
     </row>
@@ -2582,14 +2586,14 @@
       </c>
       <c r="B22" s="48" t="inlineStr">
         <is>
-          <t>Team leave calendar and upcoming approved leaves</t>
+          <t>Show clear approval details (who still needs to act)</t>
         </is>
       </c>
       <c r="C22" s="49" t="n">
-        <v>46232</v>
+        <v>46225</v>
       </c>
       <c r="D22" s="49" t="n">
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="E22" s="24">
         <f>IF(OR(C22="",D22=""),"",NETWORKDAYS(C22,D22))</f>
@@ -2610,87 +2614,87 @@
       </c>
       <c r="I22" s="48" t="inlineStr">
         <is>
-          <t>Team Leave Calendar page (month/week views, filters, leave chips) and Upcoming Approved Leaves page are both built with mock data.</t>
+          <t>Changed: progress-bar UI removed. Shared Approval Details table + ApproverStatusBadge on employee/approver/admin request pages.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="50" t="inlineStr">
-        <is>
-          <t>5. Admin Features</t>
-        </is>
-      </c>
-      <c r="B23" s="50" t="inlineStr">
-        <is>
-          <t>Admin view of leave requests and request details</t>
-        </is>
-      </c>
-      <c r="C23" s="51" t="n">
+      <c r="A23" s="48" t="inlineStr">
+        <is>
+          <t>4. Approver / Team Features</t>
+        </is>
+      </c>
+      <c r="B23" s="48" t="inlineStr">
+        <is>
+          <t>File leave on behalf of a team member</t>
+        </is>
+      </c>
+      <c r="C23" s="49" t="n">
+        <v>46226</v>
+      </c>
+      <c r="D23" s="49" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E23" s="24">
+        <f>IF(OR(C23="",D23=""),"",NETWORKDAYS(C23,D23))</f>
+        <v/>
+      </c>
+      <c r="F23" s="66" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G23" s="25">
+        <f>IF(F23="Completed",1,IF(F23="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H23" s="65">
+        <f>IF(C23="","",C23+MOD(5-WEEKDAY(C23,2),7))</f>
+        <v/>
+      </c>
+      <c r="I23" s="48" t="inlineStr">
+        <is>
+          <t>UI complete; holidays hook wired. Full live submit / member directory API still being finished.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="48" t="inlineStr">
+        <is>
+          <t>4. Approver / Team Features</t>
+        </is>
+      </c>
+      <c r="B24" s="48" t="inlineStr">
+        <is>
+          <t>Team leave calendar and upcoming approved leaves</t>
+        </is>
+      </c>
+      <c r="C24" s="49" t="n">
         <v>46232</v>
       </c>
-      <c r="D23" s="51" t="n">
+      <c r="D24" s="49" t="n">
         <v>46232</v>
       </c>
-      <c r="E23" s="27">
-        <f>IF(OR(C23="",D23=""),"",NETWORKDAYS(C23,D23))</f>
-        <v/>
-      </c>
-      <c r="F23" s="36" t="inlineStr">
+      <c r="E24" s="24">
+        <f>IF(OR(C24="",D24=""),"",NETWORKDAYS(C24,D24))</f>
+        <v/>
+      </c>
+      <c r="F24" s="36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="G23" s="28">
-        <f>IF(F23="Completed",1,IF(F23="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H23" s="66">
-        <f>IF(C23="","",C23+MOD(5-WEEKDAY(C23,2),7))</f>
-        <v/>
-      </c>
-      <c r="I23" s="50" t="inlineStr">
-        <is>
-          <t>Admin Leave Requests list (pending/all tabs, filters, search, reminders) and detail/view/validate pages are all built with mock data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="50" t="inlineStr">
-        <is>
-          <t>5. Admin Features</t>
-        </is>
-      </c>
-      <c r="B24" s="50" t="inlineStr">
-        <is>
-          <t>Review vacation-to-sick leave conversion requests</t>
-        </is>
-      </c>
-      <c r="C24" s="51" t="n">
-        <v>46232</v>
-      </c>
-      <c r="D24" s="51" t="n">
-        <v>46232</v>
-      </c>
-      <c r="E24" s="27">
-        <f>IF(OR(C24="",D24=""),"",NETWORKDAYS(C24,D24))</f>
-        <v/>
-      </c>
-      <c r="F24" s="36" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="G24" s="28">
+      <c r="G24" s="25">
         <f>IF(F24="Completed",1,IF(F24="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H24" s="66">
+      <c r="H24" s="65">
         <f>IF(C24="","",C24+MOD(5-WEEKDAY(C24,2),7))</f>
         <v/>
       </c>
-      <c r="I24" s="50" t="inlineStr">
-        <is>
-          <t>Conversion review is handled via Admin Leave Validate page; conversion state visible on request detail/view pages.</t>
+      <c r="I24" s="48" t="inlineStr">
+        <is>
+          <t>Calendar + upcoming pages built. Still on mock calendar data until team-calendar API is connected.</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2706,7 @@
       </c>
       <c r="B25" s="50" t="inlineStr">
         <is>
-          <t>Manage leave balances and credit distribution</t>
+          <t>Admin view of leave requests and request details</t>
         </is>
       </c>
       <c r="C25" s="51" t="n">
@@ -2724,13 +2728,13 @@
         <f>IF(F25="Completed",1,IF(F25="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H25" s="66">
+      <c r="H25" s="67">
         <f>IF(C25="","",C25+MOD(5-WEEKDAY(C25,2),7))</f>
         <v/>
       </c>
       <c r="I25" s="50" t="inlineStr">
         <is>
-          <t>Admin Leave Balances page with filters, adjust-credits modal, and full distribution flows (annual, newly-regularized, parental, contractual) are built with mock data.</t>
+          <t>Admin Leave Requests list + detail/validate UIs built. Still mock data until admin API wiring.</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2746,7 @@
       </c>
       <c r="B26" s="50" t="inlineStr">
         <is>
-          <t>Administrative logs</t>
+          <t>Review vacation-to-sick leave conversion requests</t>
         </is>
       </c>
       <c r="C26" s="51" t="n">
@@ -2764,13 +2768,13 @@
         <f>IF(F26="Completed",1,IF(F26="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H26" s="66">
+      <c r="H26" s="67">
         <f>IF(C26="","",C26+MOD(5-WEEKDAY(C26,2),7))</f>
         <v/>
       </c>
       <c r="I26" s="50" t="inlineStr">
         <is>
-          <t>Admin Administrative Log page with search, filters, month-year picker, sorting, and pagination is built with mock data.</t>
+          <t>Conversion review via Admin Leave Validate page (UI). Live admin conversion API not wired yet.</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2786,7 @@
       </c>
       <c r="B27" s="50" t="inlineStr">
         <is>
-          <t>Monthly Attendance Report</t>
+          <t>Manage leave balances and credit distribution</t>
         </is>
       </c>
       <c r="C27" s="51" t="n">
@@ -2804,13 +2808,13 @@
         <f>IF(F27="Completed",1,IF(F27="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H27" s="66">
+      <c r="H27" s="67">
         <f>IF(C27="","",C27+MOD(5-WEEKDAY(C27,2),7))</f>
         <v/>
       </c>
       <c r="I27" s="50" t="inlineStr">
         <is>
-          <t>Report page with month/cut-off filters, employee multi-select, group filter, calendar grid, legend, print, and download. Uses mock data.</t>
+          <t>Balances + distribution flows (annual, newly-regularized, parental, contractual) built with mock data.</t>
         </is>
       </c>
     </row>
@@ -2822,14 +2826,14 @@
       </c>
       <c r="B28" s="50" t="inlineStr">
         <is>
-          <t>Leave Monetization Candidates report</t>
+          <t>Administrative logs</t>
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="D28" s="51" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="E28" s="27">
         <f>IF(OR(C28="",D28=""),"",NETWORKDAYS(C28,D28))</f>
@@ -2844,13 +2848,13 @@
         <f>IF(F28="Completed",1,IF(F28="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H28" s="66">
+      <c r="H28" s="67">
         <f>IF(C28="","",C28+MOD(5-WEEKDAY(C28,2),7))</f>
         <v/>
       </c>
       <c r="I28" s="50" t="inlineStr">
         <is>
-          <t>Report page with year filter, eligibility filters, sortable table, summary totals, print, and download. Uses mock data.</t>
+          <t>Admin Administrative Log UI built with mock data.</t>
         </is>
       </c>
     </row>
@@ -2862,14 +2866,14 @@
       </c>
       <c r="B29" s="50" t="inlineStr">
         <is>
-          <t>Employees with LWOP report</t>
+          <t>Monthly Attendance Report</t>
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="D29" s="51" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="E29" s="27">
         <f>IF(OR(C29="",D29=""),"",NETWORKDAYS(C29,D29))</f>
@@ -2884,13 +2888,13 @@
         <f>IF(F29="Completed",1,IF(F29="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H29" s="66">
+      <c r="H29" s="67">
         <f>IF(C29="","",C29+MOD(5-WEEKDAY(C29,2),7))</f>
         <v/>
       </c>
       <c r="I29" s="50" t="inlineStr">
         <is>
-          <t>Report page with year and group filters, sortable LWOP summary table, print, and download. Uses mock data.</t>
+          <t>Report UI built (filters, grid, print/download). Mock data until reports API.</t>
         </is>
       </c>
     </row>
@@ -2902,14 +2906,14 @@
       </c>
       <c r="B30" s="50" t="inlineStr">
         <is>
-          <t>Support other leave types (emergency, maternity, etc.) in the screens</t>
+          <t>Leave Monetization Candidates report</t>
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="D30" s="51" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E30" s="27">
         <f>IF(OR(C30="",D30=""),"",NETWORKDAYS(C30,D30))</f>
@@ -2924,118 +2928,118 @@
         <f>IF(F30="Completed",1,IF(F30="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H30" s="66">
+      <c r="H30" s="67">
         <f>IF(C30="","",C30+MOD(5-WEEKDAY(C30,2),7))</f>
         <v/>
       </c>
       <c r="I30" s="50" t="inlineStr">
         <is>
-          <t>Emergency, PTB, Maternity/Paternity handled in employee/team filing and in admin screens. Monthly attendance report covers all leave categories including LWOP.</t>
+          <t>Report UI built. Mock data until reports API.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="67" t="inlineStr">
+      <c r="A31" s="50" t="inlineStr">
+        <is>
+          <t>5. Admin Features</t>
+        </is>
+      </c>
+      <c r="B31" s="50" t="inlineStr">
+        <is>
+          <t>Employees with LWOP report</t>
+        </is>
+      </c>
+      <c r="C31" s="51" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D31" s="51" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E31" s="27">
+        <f>IF(OR(C31="",D31=""),"",NETWORKDAYS(C31,D31))</f>
+        <v/>
+      </c>
+      <c r="F31" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G31" s="28">
+        <f>IF(F31="Completed",1,IF(F31="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H31" s="67">
+        <f>IF(C31="","",C31+MOD(5-WEEKDAY(C31,2),7))</f>
+        <v/>
+      </c>
+      <c r="I31" s="50" t="inlineStr">
+        <is>
+          <t>Report UI built. Mock data until reports API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="50" t="inlineStr">
+        <is>
+          <t>5. Admin Features</t>
+        </is>
+      </c>
+      <c r="B32" s="50" t="inlineStr">
+        <is>
+          <t>Support other leave types (emergency, maternity, etc.) in the screens</t>
+        </is>
+      </c>
+      <c r="C32" s="51" t="n">
+        <v>46225</v>
+      </c>
+      <c r="D32" s="51" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E32" s="27">
+        <f>IF(OR(C32="",D32=""),"",NETWORKDAYS(C32,D32))</f>
+        <v/>
+      </c>
+      <c r="F32" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G32" s="28">
+        <f>IF(F32="Completed",1,IF(F32="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H32" s="67">
+        <f>IF(C32="","",C32+MOD(5-WEEKDAY(C32,2),7))</f>
+        <v/>
+      </c>
+      <c r="I32" s="50" t="inlineStr">
+        <is>
+          <t>Emergency, PTB, Maternity/Paternity handled across filing and admin screens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="68" t="inlineStr">
         <is>
           <t>6. UI Polish &amp; Cleanup</t>
         </is>
       </c>
-      <c r="B31" s="67" t="inlineStr">
+      <c r="B33" s="68" t="inlineStr">
         <is>
           <t>Review and clean up global CSS (colors, fonts, spacing, typography)</t>
         </is>
       </c>
-      <c r="C31" s="68" t="n">
+      <c r="C33" s="69" t="n">
         <v>46233</v>
       </c>
-      <c r="D31" s="68" t="n">
-        <v>46242</v>
-      </c>
-      <c r="E31" s="30">
-        <f>IF(OR(C31="",D31=""),"",NETWORKDAYS(C31,D31))</f>
-        <v/>
-      </c>
-      <c r="F31" s="69" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G31" s="31">
-        <f>IF(F31="Completed",1,IF(F31="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H31" s="70">
-        <f>IF(C31="","",C31+MOD(5-WEEKDAY(C31,2),7))</f>
-        <v/>
-      </c>
-      <c r="I31" s="67" t="inlineStr">
-        <is>
-          <t>Currently in progress — checking index.css theme tokens, base styles, and consistency with Tailwind usage across screens.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="67" t="inlineStr">
-        <is>
-          <t>6. UI Polish &amp; Cleanup</t>
-        </is>
-      </c>
-      <c r="B32" s="67" t="inlineStr">
-        <is>
-          <t>Check and fix app shell layout (sidebar, top header, main content area)</t>
-        </is>
-      </c>
-      <c r="C32" s="68" t="n">
-        <v>46233</v>
-      </c>
-      <c r="D32" s="68" t="n">
-        <v>46242</v>
-      </c>
-      <c r="E32" s="30">
-        <f>IF(OR(C32="",D32=""),"",NETWORKDAYS(C32,D32))</f>
-        <v/>
-      </c>
-      <c r="F32" s="69" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G32" s="31">
-        <f>IF(F32="Completed",1,IF(F32="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H32" s="70">
-        <f>IF(C32="","",C32+MOD(5-WEEKDAY(C32,2),7))</f>
-        <v/>
-      </c>
-      <c r="I32" s="67" t="inlineStr">
-        <is>
-          <t>Currently in progress — reviewing AppLayout, collapsible sidebar, header alignment, and page padding/overflow behavior.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="67" t="inlineStr">
-        <is>
-          <t>6. UI Polish &amp; Cleanup</t>
-        </is>
-      </c>
-      <c r="B33" s="67" t="inlineStr">
-        <is>
-          <t>Standardize screen layouts (tables, filter bars, forms, and reports)</t>
-        </is>
-      </c>
-      <c r="C33" s="68" t="n">
-        <v>46233</v>
-      </c>
-      <c r="D33" s="68" t="n">
-        <v>46249</v>
+      <c r="D33" s="69" t="n">
+        <v>46256</v>
       </c>
       <c r="E33" s="30">
         <f>IF(OR(C33="",D33=""),"",NETWORKDAYS(C33,D33))</f>
         <v/>
       </c>
-      <c r="F33" s="69" t="inlineStr">
+      <c r="F33" s="66" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -3048,121 +3052,129 @@
         <f>IF(C33="","",C33+MOD(5-WEEKDAY(C33,2),7))</f>
         <v/>
       </c>
-      <c r="I33" s="67" t="inlineStr">
-        <is>
-          <t>Currently in progress — aligning filter control heights, table spacing, button placement, and responsive layout on list/form/report pages.</t>
+      <c r="I33" s="68" t="inlineStr">
+        <is>
+          <t>STILL IN PROGRESS as of 2026-08-13 — codebase review and CSS cleanup ongoing.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="56" t="inlineStr">
-        <is>
-          <t>7. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B34" s="56" t="inlineStr">
-        <is>
-          <t>Connect frontend to backend API (base connection and shared data types)</t>
-        </is>
-      </c>
-      <c r="C34" s="71" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D34" s="71" t="n"/>
-      <c r="E34" s="33">
+      <c r="A34" s="68" t="inlineStr">
+        <is>
+          <t>6. UI Polish &amp; Cleanup</t>
+        </is>
+      </c>
+      <c r="B34" s="68" t="inlineStr">
+        <is>
+          <t>Check and fix app shell layout (sidebar, top header, main content area)</t>
+        </is>
+      </c>
+      <c r="C34" s="69" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D34" s="69" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E34" s="30">
         <f>IF(OR(C34="",D34=""),"",NETWORKDAYS(C34,D34))</f>
         <v/>
       </c>
-      <c r="F34" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G34" s="34">
+      <c r="F34" s="66" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G34" s="31">
         <f>IF(F34="Completed",1,IF(F34="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H34" s="73">
+      <c r="H34" s="70">
         <f>IF(C34="","",C34+MOD(5-WEEKDAY(C34,2),7))</f>
         <v/>
       </c>
-      <c r="I34" s="56" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+      <c r="I34" s="68" t="inlineStr">
+        <is>
+          <t>STILL IN PROGRESS as of 2026-08-13 — AppLayout, sidebar, header, overflow, and content spacing under review.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="56" t="inlineStr">
-        <is>
-          <t>7. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B35" s="56" t="inlineStr">
-        <is>
-          <t>Use portal cookies / session to identify the user (no separate login page)</t>
-        </is>
-      </c>
-      <c r="C35" s="71" t="n">
-        <v>46226</v>
-      </c>
-      <c r="D35" s="71" t="n"/>
-      <c r="E35" s="33">
+      <c r="A35" s="68" t="inlineStr">
+        <is>
+          <t>6. UI Polish &amp; Cleanup</t>
+        </is>
+      </c>
+      <c r="B35" s="68" t="inlineStr">
+        <is>
+          <t>Standardize screen layouts (tables, filter bars, forms, and reports)</t>
+        </is>
+      </c>
+      <c r="C35" s="69" t="n">
+        <v>46233</v>
+      </c>
+      <c r="D35" s="69" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E35" s="30">
         <f>IF(OR(C35="",D35=""),"",NETWORKDAYS(C35,D35))</f>
         <v/>
       </c>
-      <c r="F35" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G35" s="34">
+      <c r="F35" s="66" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G35" s="31">
         <f>IF(F35="Completed",1,IF(F35="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H35" s="73">
+      <c r="H35" s="70">
         <f>IF(C35="","",C35+MOD(5-WEEKDAY(C35,2),7))</f>
         <v/>
       </c>
-      <c r="I35" s="56" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known. Agreed with backend: cookies/session — no login screen.</t>
+      <c r="I35" s="68" t="inlineStr">
+        <is>
+          <t>STILL IN PROGRESS as of 2026-08-13 — table/filter/form consistency and empty states being aligned across pages.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="56" t="inlineStr">
-        <is>
-          <t>7. Backend Integration (TBD)</t>
-        </is>
-      </c>
-      <c r="B36" s="56" t="inlineStr">
-        <is>
-          <t>Connect employee leave screens to live API (file, history, cancel, edit)</t>
-        </is>
-      </c>
-      <c r="C36" s="71" t="n"/>
-      <c r="D36" s="71" t="n"/>
-      <c r="E36" s="33">
+      <c r="A36" s="68" t="inlineStr">
+        <is>
+          <t>6. UI Polish &amp; Cleanup</t>
+        </is>
+      </c>
+      <c r="B36" s="68" t="inlineStr">
+        <is>
+          <t>Extract shared leave UI and remove unused placeholder code</t>
+        </is>
+      </c>
+      <c r="C36" s="69" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D36" s="69" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E36" s="30">
         <f>IF(OR(C36="",D36=""),"",NETWORKDAYS(C36,D36))</f>
         <v/>
       </c>
-      <c r="F36" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G36" s="34">
+      <c r="F36" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G36" s="31">
         <f>IF(F36="Completed",1,IF(F36="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H36" s="73">
+      <c r="H36" s="70">
         <f>IF(C36="","",C36+MOD(5-WEEKDAY(C36,2),7))</f>
         <v/>
       </c>
-      <c r="I36" s="56" t="inlineStr">
-        <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+      <c r="I36" s="68" t="inlineStr">
+        <is>
+          <t>Shared leave components added; PagePlaceholder removed; EmptyState / TableEmptyRow rolled out.</t>
         </is>
       </c>
     </row>
@@ -3174,31 +3186,35 @@
       </c>
       <c r="B37" s="56" t="inlineStr">
         <is>
-          <t>Connect approver / team screens to live API (inbox, approve, reject)</t>
-        </is>
-      </c>
-      <c r="C37" s="71" t="n"/>
-      <c r="D37" s="71" t="n"/>
+          <t>Connect frontend to backend API (base connection and shared data types)</t>
+        </is>
+      </c>
+      <c r="C37" s="71" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D37" s="71" t="n">
+        <v>46247</v>
+      </c>
       <c r="E37" s="33">
         <f>IF(OR(C37="",D37=""),"",NETWORKDAYS(C37,D37))</f>
         <v/>
       </c>
-      <c r="F37" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F37" s="36" t="inlineStr">
+        <is>
+          <t>Completed</t>
         </is>
       </c>
       <c r="G37" s="34">
         <f>IF(F37="Completed",1,IF(F37="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H37" s="73">
+      <c r="H37" s="72">
         <f>IF(C37="","",C37+MOD(5-WEEKDAY(C37,2),7))</f>
         <v/>
       </c>
       <c r="I37" s="56" t="inlineStr">
         <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+          <t>Axios client (/api), ApiError + 401 handling, typed API modules, and SWR provider/hooks are in place.</t>
         </is>
       </c>
     </row>
@@ -3210,31 +3226,35 @@
       </c>
       <c r="B38" s="56" t="inlineStr">
         <is>
-          <t>Connect admin screens to live API (balances, conversion, reports)</t>
-        </is>
-      </c>
-      <c r="C38" s="71" t="n"/>
-      <c r="D38" s="71" t="n"/>
+          <t>Use portal cookies / session to identify the user (no separate login page)</t>
+        </is>
+      </c>
+      <c r="C38" s="71" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D38" s="71" t="n">
+        <v>46247</v>
+      </c>
       <c r="E38" s="33">
         <f>IF(OR(C38="",D38=""),"",NETWORKDAYS(C38,D38))</f>
         <v/>
       </c>
-      <c r="F38" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F38" s="66" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G38" s="34">
         <f>IF(F38="Completed",1,IF(F38="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H38" s="73">
+      <c r="H38" s="72">
         <f>IF(C38="","",C38+MOD(5-WEEKDAY(C38,2),7))</f>
         <v/>
       </c>
       <c r="I38" s="56" t="inlineStr">
         <is>
-          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
+          <t>Auth bootstraps from userID cookie + GET /api/me. Dev-only Employee ID entry (/login) for local testing — production remains cookie/portal session.</t>
         </is>
       </c>
     </row>
@@ -3246,145 +3266,147 @@
       </c>
       <c r="B39" s="56" t="inlineStr">
         <is>
-          <t>Joint frontend–backend smoke check once APIs are available</t>
-        </is>
-      </c>
-      <c r="C39" s="71" t="n"/>
-      <c r="D39" s="71" t="n"/>
+          <t>Connect employee leave screens to live API (file, history, cancel, edit)</t>
+        </is>
+      </c>
+      <c r="C39" s="71" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D39" s="71" t="n">
+        <v>46247</v>
+      </c>
       <c r="E39" s="33">
         <f>IF(OR(C39="",D39=""),"",NETWORKDAYS(C39,D39))</f>
         <v/>
       </c>
-      <c r="F39" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F39" s="66" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G39" s="34">
         <f>IF(F39="Completed",1,IF(F39="In Progress",0.5,0))</f>
         <v/>
       </c>
-      <c r="H39" s="73">
+      <c r="H39" s="72">
         <f>IF(C39="","",C39+MOD(5-WEEKDAY(C39,2),7))</f>
         <v/>
       </c>
       <c r="I39" s="56" t="inlineStr">
         <is>
+          <t>Dashboard, activity log, file/edit/cancel/convert, and details are on live APIs. Continue hardening error handling and edge cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B40" s="56" t="inlineStr">
+        <is>
+          <t>Connect approver / team screens to live API (inbox, approve, reject)</t>
+        </is>
+      </c>
+      <c r="C40" s="71" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D40" s="71" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E40" s="33">
+        <f>IF(OR(C40="",D40=""),"",NETWORKDAYS(C40,D40))</f>
+        <v/>
+      </c>
+      <c r="F40" s="66" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G40" s="34">
+        <f>IF(F40="Completed",1,IF(F40="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H40" s="72">
+        <f>IF(C40="","",C40+MOD(5-WEEKDAY(C40,2),7))</f>
+        <v/>
+      </c>
+      <c r="I40" s="56" t="inlineStr">
+        <is>
+          <t>Approvals inbox + approve/reject live. Team calendar / file-for-member still need fuller API coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B41" s="56" t="inlineStr">
+        <is>
+          <t>Connect admin screens to live API (balances, conversion, reports)</t>
+        </is>
+      </c>
+      <c r="C41" s="71" t="n"/>
+      <c r="D41" s="71" t="n"/>
+      <c r="E41" s="33">
+        <f>IF(OR(C41="",D41=""),"",NETWORKDAYS(C41,D41))</f>
+        <v/>
+      </c>
+      <c r="F41" s="73" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G41" s="34">
+        <f>IF(F41="Completed",1,IF(F41="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H41" s="72">
+        <f>IF(C41="","",C41+MOD(5-WEEKDAY(C41,2),7))</f>
+        <v/>
+      </c>
+      <c r="I41" s="56" t="inlineStr">
+        <is>
+          <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known. Admin screens still use mock data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="56" t="inlineStr">
+        <is>
+          <t>7. Backend Integration (TBD)</t>
+        </is>
+      </c>
+      <c r="B42" s="56" t="inlineStr">
+        <is>
+          <t>Joint frontend–backend smoke check once APIs are available</t>
+        </is>
+      </c>
+      <c r="C42" s="71" t="n"/>
+      <c r="D42" s="71" t="n"/>
+      <c r="E42" s="33">
+        <f>IF(OR(C42="",D42=""),"",NETWORKDAYS(C42,D42))</f>
+        <v/>
+      </c>
+      <c r="F42" s="73" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G42" s="34">
+        <f>IF(F42="Completed",1,IF(F42="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H42" s="72">
+        <f>IF(C42="","",C42+MOD(5-WEEKDAY(C42,2),7))</f>
+        <v/>
+      </c>
+      <c r="I42" s="56" t="inlineStr">
+        <is>
           <t>Duration TBD — frontend and backend work separately. Update Start/End when schedule is known.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="57" t="inlineStr">
-        <is>
-          <t>8. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B40" s="57" t="inlineStr">
-        <is>
-          <t>Employee flow testing (file, edit, cancel, view history)</t>
-        </is>
-      </c>
-      <c r="C40" s="74" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D40" s="74" t="n"/>
-      <c r="E40" s="36">
-        <f>IF(OR(C40="",D40=""),"",NETWORKDAYS(C40,D40))</f>
-        <v/>
-      </c>
-      <c r="F40" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G40" s="37">
-        <f>IF(F40="Completed",1,IF(F40="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H40" s="75">
-        <f>IF(C40="","",C40+MOD(5-WEEKDAY(C40,2),7))</f>
-        <v/>
-      </c>
-      <c r="I40" s="57" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="57" t="inlineStr">
-        <is>
-          <t>8. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B41" s="57" t="inlineStr">
-        <is>
-          <t>Approver flow testing (approve, reject, team views)</t>
-        </is>
-      </c>
-      <c r="C41" s="74" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D41" s="74" t="n"/>
-      <c r="E41" s="36">
-        <f>IF(OR(C41="",D41=""),"",NETWORKDAYS(C41,D41))</f>
-        <v/>
-      </c>
-      <c r="F41" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G41" s="37">
-        <f>IF(F41="Completed",1,IF(F41="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H41" s="75">
-        <f>IF(C41="","",C41+MOD(5-WEEKDAY(C41,2),7))</f>
-        <v/>
-      </c>
-      <c r="I41" s="57" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="57" t="inlineStr">
-        <is>
-          <t>8. Testing (after development)</t>
-        </is>
-      </c>
-      <c r="B42" s="57" t="inlineStr">
-        <is>
-          <t>Admin flow testing (balances, conversion, reports)</t>
-        </is>
-      </c>
-      <c r="C42" s="74" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D42" s="74" t="n"/>
-      <c r="E42" s="36">
-        <f>IF(OR(C42="",D42=""),"",NETWORKDAYS(C42,D42))</f>
-        <v/>
-      </c>
-      <c r="F42" s="72" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G42" s="37">
-        <f>IF(F42="Completed",1,IF(F42="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H42" s="75">
-        <f>IF(C42="","",C42+MOD(5-WEEKDAY(C42,2),7))</f>
-        <v/>
-      </c>
-      <c r="I42" s="57" t="inlineStr">
-        <is>
-          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3418,7 @@
       </c>
       <c r="B43" s="57" t="inlineStr">
         <is>
-          <t>Mobile / responsive check on common screens</t>
+          <t>Employee flow testing (file, edit, cancel, view history)</t>
         </is>
       </c>
       <c r="C43" s="74" t="n">
@@ -3407,7 +3429,7 @@
         <f>IF(OR(C43="",D43=""),"",NETWORKDAYS(C43,D43))</f>
         <v/>
       </c>
-      <c r="F43" s="72" t="inlineStr">
+      <c r="F43" s="73" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3434,7 +3456,7 @@
       </c>
       <c r="B44" s="57" t="inlineStr">
         <is>
-          <t>Fix issues found during testing</t>
+          <t>Approver flow testing (approve, reject, team views)</t>
         </is>
       </c>
       <c r="C44" s="74" t="n">
@@ -3445,7 +3467,7 @@
         <f>IF(OR(C44="",D44=""),"",NETWORKDAYS(C44,D44))</f>
         <v/>
       </c>
-      <c r="F44" s="72" t="inlineStr">
+      <c r="F44" s="73" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -3465,132 +3487,246 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="58" t="inlineStr">
+      <c r="A45" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B45" s="57" t="inlineStr">
+        <is>
+          <t>Admin flow testing (balances, conversion, reports)</t>
+        </is>
+      </c>
+      <c r="C45" s="74" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D45" s="74" t="n"/>
+      <c r="E45" s="36">
+        <f>IF(OR(C45="",D45=""),"",NETWORKDAYS(C45,D45))</f>
+        <v/>
+      </c>
+      <c r="F45" s="73" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G45" s="37">
+        <f>IF(F45="Completed",1,IF(F45="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H45" s="75">
+        <f>IF(C45="","",C45+MOD(5-WEEKDAY(C45,2),7))</f>
+        <v/>
+      </c>
+      <c r="I45" s="57" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B46" s="57" t="inlineStr">
+        <is>
+          <t>Mobile / responsive check on common screens</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D46" s="74" t="n"/>
+      <c r="E46" s="36">
+        <f>IF(OR(C46="",D46=""),"",NETWORKDAYS(C46,D46))</f>
+        <v/>
+      </c>
+      <c r="F46" s="73" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G46" s="37">
+        <f>IF(F46="Completed",1,IF(F46="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H46" s="75">
+        <f>IF(C46="","",C46+MOD(5-WEEKDAY(C46,2),7))</f>
+        <v/>
+      </c>
+      <c r="I46" s="57" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="57" t="inlineStr">
+        <is>
+          <t>8. Testing (after development)</t>
+        </is>
+      </c>
+      <c r="B47" s="57" t="inlineStr">
+        <is>
+          <t>Fix issues found during testing</t>
+        </is>
+      </c>
+      <c r="C47" s="74" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D47" s="74" t="n"/>
+      <c r="E47" s="36">
+        <f>IF(OR(C47="",D47=""),"",NETWORKDAYS(C47,D47))</f>
+        <v/>
+      </c>
+      <c r="F47" s="73" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G47" s="37">
+        <f>IF(F47="Completed",1,IF(F47="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H47" s="75">
+        <f>IF(C47="","",C47+MOD(5-WEEKDAY(C47,2),7))</f>
+        <v/>
+      </c>
+      <c r="I47" s="57" t="inlineStr">
+        <is>
+          <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="58" t="inlineStr">
         <is>
           <t>9. Documentation (after development)</t>
         </is>
       </c>
-      <c r="B45" s="58" t="inlineStr">
+      <c r="B48" s="58" t="inlineStr">
         <is>
           <t>Finalize frontend guide for the team (FRONTEND.md)</t>
         </is>
       </c>
-      <c r="C45" s="76" t="n">
+      <c r="C48" s="76" t="n">
         <v>46266</v>
       </c>
-      <c r="D45" s="76" t="n"/>
-      <c r="E45" s="39">
-        <f>IF(OR(C45="",D45=""),"",NETWORKDAYS(C45,D45))</f>
-        <v/>
-      </c>
-      <c r="F45" s="72" t="inlineStr">
+      <c r="D48" s="76" t="n"/>
+      <c r="E48" s="39">
+        <f>IF(OR(C48="",D48=""),"",NETWORKDAYS(C48,D48))</f>
+        <v/>
+      </c>
+      <c r="F48" s="73" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G45" s="40">
-        <f>IF(F45="Completed",1,IF(F45="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H45" s="77">
-        <f>IF(C45="","",C45+MOD(5-WEEKDAY(C45,2),7))</f>
-        <v/>
-      </c>
-      <c r="I45" s="58" t="inlineStr">
+      <c r="G48" s="40">
+        <f>IF(F48="Completed",1,IF(F48="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H48" s="77">
+        <f>IF(C48="","",C48+MOD(5-WEEKDAY(C48,2),7))</f>
+        <v/>
+      </c>
+      <c r="I48" s="58" t="inlineStr">
         <is>
           <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="58" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="58" t="inlineStr">
         <is>
           <t>9. Documentation (after development)</t>
         </is>
       </c>
-      <c r="B46" s="58" t="inlineStr">
+      <c r="B49" s="58" t="inlineStr">
         <is>
           <t>Prepare short demo / walkthrough notes for stakeholders</t>
         </is>
       </c>
-      <c r="C46" s="76" t="n">
+      <c r="C49" s="76" t="n">
         <v>46266</v>
       </c>
-      <c r="D46" s="76" t="n"/>
-      <c r="E46" s="39">
-        <f>IF(OR(C46="",D46=""),"",NETWORKDAYS(C46,D46))</f>
-        <v/>
-      </c>
-      <c r="F46" s="72" t="inlineStr">
+      <c r="D49" s="76" t="n"/>
+      <c r="E49" s="39">
+        <f>IF(OR(C49="",D49=""),"",NETWORKDAYS(C49,D49))</f>
+        <v/>
+      </c>
+      <c r="F49" s="73" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G46" s="40">
-        <f>IF(F46="Completed",1,IF(F46="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H46" s="77">
-        <f>IF(C46="","",C46+MOD(5-WEEKDAY(C46,2),7))</f>
-        <v/>
-      </c>
-      <c r="I46" s="58" t="inlineStr">
+      <c r="G49" s="40">
+        <f>IF(F49="Completed",1,IF(F49="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H49" s="77">
+        <f>IF(C49="","",C49+MOD(5-WEEKDAY(C49,2),7))</f>
+        <v/>
+      </c>
+      <c r="I49" s="58" t="inlineStr">
         <is>
           <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="58" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="58" t="inlineStr">
         <is>
           <t>9. Documentation (after development)</t>
         </is>
       </c>
-      <c r="B47" s="58" t="inlineStr">
+      <c r="B50" s="58" t="inlineStr">
         <is>
           <t>Handover checklist (how to run, deploy, and who owns what)</t>
         </is>
       </c>
-      <c r="C47" s="76" t="n">
+      <c r="C50" s="76" t="n">
         <v>46266</v>
       </c>
-      <c r="D47" s="76" t="n"/>
-      <c r="E47" s="39">
-        <f>IF(OR(C47="",D47=""),"",NETWORKDAYS(C47,D47))</f>
-        <v/>
-      </c>
-      <c r="F47" s="72" t="inlineStr">
+      <c r="D50" s="76" t="n"/>
+      <c r="E50" s="39">
+        <f>IF(OR(C50="",D50=""),"",NETWORKDAYS(C50,D50))</f>
+        <v/>
+      </c>
+      <c r="F50" s="73" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="G47" s="40">
-        <f>IF(F47="Completed",1,IF(F47="In Progress",0.5,0))</f>
-        <v/>
-      </c>
-      <c r="H47" s="77">
-        <f>IF(C47="","",C47+MOD(5-WEEKDAY(C47,2),7))</f>
-        <v/>
-      </c>
-      <c r="I47" s="58" t="inlineStr">
+      <c r="G50" s="40">
+        <f>IF(F50="Completed",1,IF(F50="In Progress",0.5,0))</f>
+        <v/>
+      </c>
+      <c r="H50" s="77">
+        <f>IF(C50="","",C50+MOD(5-WEEKDAY(C50,2),7))</f>
+        <v/>
+      </c>
+      <c r="I50" s="58" t="inlineStr">
         <is>
           <t>Starts after development. End of August commitment covers development only — dates TBD.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Commitment: frontend DEVELOPMENT finished by end of August (weekdays = NETWORKDAYS). Backend Integration has TBD end dates (teams work separately — fill dates when known). Testing and Documentation start after development (from Sep 2026); end dates TBD. No login page — portal cookies/session with backend.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I47"/>
+  <autoFilter ref="A1:I50"/>
   <mergeCells count="1">
-    <mergeCell ref="A49:I49"/>
+    <mergeCell ref="A52:I52"/>
   </mergeCells>
-  <conditionalFormatting sqref="G2:G47">
+  <conditionalFormatting sqref="G2:G50">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -3603,7 +3739,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Completed,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3657,7 +3793,7 @@
     <row r="6">
       <c r="A6" s="78" t="inlineStr">
         <is>
-          <t>Backend Integration is listed with TBD dates — teams work separately for now.</t>
+          <t>Backend Integration is underway (employee + key approver). Admin APIs and remaining team screens still TBD.</t>
         </is>
       </c>
     </row>

</xml_diff>